<commit_message>
🏆 Expert Rankings Updated — 15 Sep 2026 20:20 IST
</commit_message>
<xml_diff>
--- a/output/MF_Expert_Rankings.xlsx
+++ b/output/MF_Expert_Rankings.xlsx
@@ -617,7 +617,7 @@
     <row r="1" ht="50" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>🏆  MF EXPERT RANKINGS  |  Generated: 14 Sep 2026 21:00</t>
+          <t>🏆  MF EXPERT RANKINGS  |  Generated: 15 Sep 2026 20:19</t>
         </is>
       </c>
     </row>
@@ -1242,7 +1242,7 @@
         <v>-0.42</v>
       </c>
       <c r="H32" s="7" t="n">
-        <v>8427847910015416</v>
+        <v>8427847910015000</v>
       </c>
     </row>
     <row r="33">
@@ -51489,7 +51489,7 @@
         <v>-13.7</v>
       </c>
       <c r="T3" s="11" t="n">
-        <v>8427847910015416</v>
+        <v>8427847910015000</v>
       </c>
       <c r="U3" s="18" t="n">
         <v>11.604</v>

</xml_diff>

<commit_message>
🏆 Expert Rankings Updated — 16 Sep 2026 20:17 IST
</commit_message>
<xml_diff>
--- a/output/MF_Expert_Rankings.xlsx
+++ b/output/MF_Expert_Rankings.xlsx
@@ -617,7 +617,7 @@
     <row r="1" ht="50" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>🏆  MF EXPERT RANKINGS  |  Generated: 15 Sep 2026 20:19</t>
+          <t>🏆  MF EXPERT RANKINGS  |  Generated: 16 Sep 2026 20:17</t>
         </is>
       </c>
     </row>
@@ -1242,7 +1242,7 @@
         <v>-0.42</v>
       </c>
       <c r="H32" s="7" t="n">
-        <v>8427847910015000</v>
+        <v>8427847910015416</v>
       </c>
     </row>
     <row r="33">
@@ -51489,7 +51489,7 @@
         <v>-13.7</v>
       </c>
       <c r="T3" s="11" t="n">
-        <v>8427847910015000</v>
+        <v>8427847910015416</v>
       </c>
       <c r="U3" s="18" t="n">
         <v>11.604</v>

</xml_diff>

<commit_message>
🏆 Expert Rankings Updated — 23 Sep 2026 20:32 IST
</commit_message>
<xml_diff>
--- a/output/MF_Expert_Rankings.xlsx
+++ b/output/MF_Expert_Rankings.xlsx
@@ -617,7 +617,7 @@
     <row r="1" ht="50" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>🏆  MF EXPERT RANKINGS  |  Generated: 22 Sep 2026 20:17</t>
+          <t>🏆  MF EXPERT RANKINGS  |  Generated: 23 Sep 2026 20:32</t>
         </is>
       </c>
     </row>
@@ -1242,7 +1242,7 @@
         <v>-0.42</v>
       </c>
       <c r="H32" s="7" t="n">
-        <v>8427847910015416</v>
+        <v>8427847910015000</v>
       </c>
     </row>
     <row r="33">
@@ -51489,7 +51489,7 @@
         <v>-13.7</v>
       </c>
       <c r="T3" s="11" t="n">
-        <v>8427847910015416</v>
+        <v>8427847910015000</v>
       </c>
       <c r="U3" s="18" t="n">
         <v>11.604</v>

</xml_diff>

<commit_message>
🏆 Expert Rankings Updated — 01 Oct 2026 21:53 IST
</commit_message>
<xml_diff>
--- a/output/MF_Expert_Rankings.xlsx
+++ b/output/MF_Expert_Rankings.xlsx
@@ -617,7 +617,7 @@
     <row r="1" ht="50" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>🏆  MF EXPERT RANKINGS  |  Generated: 30 Sep 2026 21:29</t>
+          <t>🏆  MF EXPERT RANKINGS  |  Generated: 01 Oct 2026 21:53</t>
         </is>
       </c>
     </row>
@@ -1242,7 +1242,7 @@
         <v>-0.42</v>
       </c>
       <c r="H32" s="6" t="n">
-        <v>8427847910015416</v>
+        <v>8427847910015000</v>
       </c>
     </row>
     <row r="33">
@@ -56431,7 +56431,7 @@
         <v>-13.7</v>
       </c>
       <c r="T3" s="11" t="n">
-        <v>8427847910015416</v>
+        <v>8427847910015000</v>
       </c>
       <c r="U3" s="18" t="n">
         <v>11.604</v>

</xml_diff>

<commit_message>
🏆 Expert Rankings Updated — 05 Oct 2026 23:14 IST
</commit_message>
<xml_diff>
--- a/output/MF_Expert_Rankings.xlsx
+++ b/output/MF_Expert_Rankings.xlsx
@@ -617,7 +617,7 @@
     <row r="1" ht="50" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>🏆  MF EXPERT RANKINGS  |  Generated: 02 Oct 2026 21:23</t>
+          <t>🏆  MF EXPERT RANKINGS  |  Generated: 05 Oct 2026 23:14</t>
         </is>
       </c>
     </row>
@@ -667,22 +667,22 @@
         </is>
       </c>
       <c r="C5" s="8" t="n">
-        <v>65.8</v>
+        <v>65.3</v>
       </c>
       <c r="D5" s="9" t="n">
-        <v>12.78</v>
+        <v>12.6</v>
       </c>
       <c r="E5" s="9" t="n">
-        <v>12.59</v>
+        <v>12.3</v>
       </c>
       <c r="F5" s="9" t="n">
-        <v>0.73</v>
+        <v>0.71</v>
       </c>
       <c r="G5" s="10" t="n">
         <v>-35.74</v>
       </c>
       <c r="H5" s="11" t="n">
-        <v>9.33</v>
+        <v>9.380000000000001</v>
       </c>
     </row>
     <row r="6">
@@ -898,22 +898,22 @@
         </is>
       </c>
       <c r="C15" s="12" t="n">
-        <v>59.5</v>
+        <v>59</v>
       </c>
       <c r="D15" s="5" t="n">
-        <v>10.2</v>
+        <v>10</v>
       </c>
       <c r="E15" s="5" t="n">
-        <v>10.4</v>
+        <v>10.21</v>
       </c>
       <c r="F15" s="5" t="n">
-        <v>0.71</v>
+        <v>0.67</v>
       </c>
       <c r="G15" s="5" t="n">
         <v>-26.35</v>
       </c>
       <c r="H15" s="6" t="n">
-        <v>7.96</v>
+        <v>7.88</v>
       </c>
     </row>
     <row r="17">
@@ -1083,13 +1083,13 @@
         <v>56.4</v>
       </c>
       <c r="D25" s="5" t="n">
-        <v>7</v>
+        <v>6.99</v>
       </c>
       <c r="E25" s="5" t="n">
-        <v>6.41</v>
+        <v>6.42</v>
       </c>
       <c r="F25" s="5" t="n">
-        <v>-13.29</v>
+        <v>-13.31</v>
       </c>
       <c r="G25" s="5" t="n">
         <v>-0.15</v>
@@ -1139,13 +1139,13 @@
         <v>53.1</v>
       </c>
       <c r="D27" s="5" t="n">
-        <v>6.96</v>
+        <v>6.95</v>
       </c>
       <c r="E27" s="5" t="n">
         <v>6.38</v>
       </c>
       <c r="F27" s="5" t="n">
-        <v>-13.95</v>
+        <v>-13.97</v>
       </c>
       <c r="G27" s="5" t="n">
         <v>-0.23</v>
@@ -1167,13 +1167,13 @@
         <v>53</v>
       </c>
       <c r="D28" s="9" t="n">
-        <v>6.92</v>
+        <v>6.91</v>
       </c>
       <c r="E28" s="9" t="n">
-        <v>6.35</v>
+        <v>6.36</v>
       </c>
       <c r="F28" s="9" t="n">
-        <v>-13.04</v>
+        <v>-13.06</v>
       </c>
       <c r="G28" s="9" t="n">
         <v>-0.18</v>
@@ -1198,10 +1198,10 @@
         <v>6.93</v>
       </c>
       <c r="E29" s="5" t="n">
-        <v>6.36</v>
+        <v>6.37</v>
       </c>
       <c r="F29" s="5" t="n">
-        <v>-9.35</v>
+        <v>-9.359999999999999</v>
       </c>
       <c r="G29" s="5" t="n">
         <v>-0.26</v>
@@ -1242,7 +1242,7 @@
         <v>-0.42</v>
       </c>
       <c r="H32" s="6" t="n">
-        <v>8427847910015416</v>
+        <v>8427847910015000</v>
       </c>
     </row>
     <row r="33">
@@ -2168,10 +2168,10 @@
         <v>76.3</v>
       </c>
       <c r="D76" s="5" t="n">
-        <v>30.57</v>
+        <v>30.62</v>
       </c>
       <c r="E76" s="5" t="n">
-        <v>18.49</v>
+        <v>18.52</v>
       </c>
       <c r="F76" s="5" t="n">
         <v>1.66</v>
@@ -2180,7 +2180,7 @@
         <v>-27.61</v>
       </c>
       <c r="H76" s="6" t="n">
-        <v>35.83</v>
+        <v>35.94</v>
       </c>
     </row>
     <row r="78">
@@ -7566,22 +7566,22 @@
         <v>76.3</v>
       </c>
       <c r="D7" s="11" t="n">
-        <v>24.52</v>
+        <v>24.12</v>
       </c>
       <c r="E7" s="11" t="n">
-        <v>30.57</v>
+        <v>30.62</v>
       </c>
       <c r="F7" s="11" t="n">
-        <v>18.49</v>
+        <v>18.52</v>
       </c>
       <c r="G7" s="11" t="n">
-        <v>8.85</v>
+        <v>8.869999999999999</v>
       </c>
       <c r="H7" s="11" t="n">
-        <v>28.57</v>
+        <v>28.61</v>
       </c>
       <c r="I7" s="11" t="n">
-        <v>27.49</v>
+        <v>27.51</v>
       </c>
       <c r="J7" s="11" t="n">
         <v>27.49</v>
@@ -7594,7 +7594,7 @@
         <v>2.24</v>
       </c>
       <c r="N7" s="9" t="n">
-        <v>18.69</v>
+        <v>18.68</v>
       </c>
       <c r="O7" s="10" t="n">
         <v>-27.61</v>
@@ -7609,19 +7609,19 @@
         <v>33.8</v>
       </c>
       <c r="S7" s="17" t="n">
-        <v>19.9</v>
+        <v>19.7</v>
       </c>
       <c r="T7" s="11" t="n">
-        <v>35.83</v>
+        <v>35.94</v>
       </c>
       <c r="U7" s="18" t="n">
         <v>0.237</v>
       </c>
       <c r="V7" s="18" t="n">
-        <v>0.028</v>
+        <v>0.027</v>
       </c>
       <c r="W7" s="11" t="n">
-        <v>1.28</v>
+        <v>1.29</v>
       </c>
       <c r="X7" s="17" t="n">
         <v>95.8</v>
@@ -7630,7 +7630,7 @@
         <v>4.6</v>
       </c>
       <c r="Z7" s="7" t="n">
-        <v>23.4794</v>
+        <v>23.5074</v>
       </c>
     </row>
     <row r="8">
@@ -7807,25 +7807,25 @@
         </is>
       </c>
       <c r="C10" s="29" t="n">
-        <v>73.7</v>
+        <v>73.8</v>
       </c>
       <c r="D10" s="22" t="n">
-        <v>16.34</v>
+        <v>15.94</v>
       </c>
       <c r="E10" s="22" t="n">
-        <v>21.71</v>
+        <v>21.66</v>
       </c>
       <c r="F10" s="22" t="n">
-        <v>12.43</v>
+        <v>12.78</v>
       </c>
       <c r="G10" s="22" t="n">
-        <v>16.46</v>
+        <v>16.44</v>
       </c>
       <c r="H10" s="22" t="n">
-        <v>17.68</v>
+        <v>17.56</v>
       </c>
       <c r="I10" s="22" t="n">
-        <v>17.34</v>
+        <v>17.28</v>
       </c>
       <c r="J10" s="22" t="n">
         <v>16.68</v>
@@ -7837,16 +7837,16 @@
         <v>1.16</v>
       </c>
       <c r="M10" s="23" t="n">
-        <v>1.58</v>
+        <v>1.57</v>
       </c>
       <c r="N10" s="23" t="n">
-        <v>15.81</v>
+        <v>15.8</v>
       </c>
       <c r="O10" s="21" t="n">
         <v>-30.78</v>
       </c>
       <c r="P10" s="23" t="n">
-        <v>0.71</v>
+        <v>0.7</v>
       </c>
       <c r="Q10" s="23" t="n">
         <v>-1.48</v>
@@ -7855,10 +7855,10 @@
         <v>16.4</v>
       </c>
       <c r="S10" s="24" t="n">
-        <v>4.7</v>
+        <v>4.8</v>
       </c>
       <c r="T10" s="22" t="n">
-        <v>24.11</v>
+        <v>24.05</v>
       </c>
       <c r="U10" s="25" t="n">
         <v>0.103</v>
@@ -7867,7 +7867,7 @@
         <v>0.008</v>
       </c>
       <c r="W10" s="22" t="n">
-        <v>0.83</v>
+        <v>0.84</v>
       </c>
       <c r="X10" s="24" t="n">
         <v>89.09999999999999</v>
@@ -7876,7 +7876,7 @@
         <v>11.2</v>
       </c>
       <c r="Z10" s="19" t="n">
-        <v>48.0052</v>
+        <v>47.9399</v>
       </c>
     </row>
     <row r="11">
@@ -8135,40 +8135,40 @@
         </is>
       </c>
       <c r="C14" s="29" t="n">
-        <v>70.90000000000001</v>
+        <v>71.2</v>
       </c>
       <c r="D14" s="22" t="n">
-        <v>28.34</v>
+        <v>28.27</v>
       </c>
       <c r="E14" s="22" t="n">
-        <v>28.02</v>
+        <v>28.14</v>
       </c>
       <c r="F14" s="22" t="n">
-        <v>10.76</v>
+        <v>11.34</v>
       </c>
       <c r="G14" s="22" t="n">
-        <v>4.91</v>
+        <v>4.94</v>
       </c>
       <c r="H14" s="22" t="n">
-        <v>26.51</v>
+        <v>26.66</v>
       </c>
       <c r="I14" s="22" t="n">
-        <v>21.68</v>
+        <v>21.79</v>
       </c>
       <c r="J14" s="22" t="n">
-        <v>15.38</v>
+        <v>15.39</v>
       </c>
       <c r="K14" s="22" t="n">
         <v>16.33</v>
       </c>
       <c r="L14" s="23" t="n">
-        <v>1.45</v>
+        <v>1.46</v>
       </c>
       <c r="M14" s="23" t="n">
-        <v>2.05</v>
+        <v>2.06</v>
       </c>
       <c r="N14" s="23" t="n">
-        <v>18.34</v>
+        <v>18.32</v>
       </c>
       <c r="O14" s="21" t="n">
         <v>-39.98</v>
@@ -8183,19 +8183,19 @@
         <v>29.5</v>
       </c>
       <c r="S14" s="24" t="n">
-        <v>19.4</v>
+        <v>19.1</v>
       </c>
       <c r="T14" s="22" t="n">
-        <v>32.15</v>
+        <v>32.32</v>
       </c>
       <c r="U14" s="25" t="n">
-        <v>0.201</v>
+        <v>0.2</v>
       </c>
       <c r="V14" s="25" t="n">
         <v>0.021</v>
       </c>
       <c r="W14" s="22" t="n">
-        <v>1.19</v>
+        <v>1.21</v>
       </c>
       <c r="X14" s="24" t="n">
         <v>82.5</v>
@@ -8204,7 +8204,7 @@
         <v>5.2</v>
       </c>
       <c r="Z14" s="19" t="n">
-        <v>16.1871</v>
+        <v>16.2323</v>
       </c>
     </row>
     <row r="15">
@@ -8217,25 +8217,25 @@
         </is>
       </c>
       <c r="C15" s="28" t="n">
-        <v>70.5</v>
+        <v>70.59999999999999</v>
       </c>
       <c r="D15" s="11" t="n">
-        <v>36.05</v>
+        <v>35.92</v>
       </c>
       <c r="E15" s="11" t="n">
-        <v>28.16</v>
+        <v>28.27</v>
       </c>
       <c r="F15" s="11" t="n">
-        <v>12.96</v>
+        <v>13.19</v>
       </c>
       <c r="G15" s="11" t="n">
-        <v>11.73</v>
+        <v>11.76</v>
       </c>
       <c r="H15" s="11" t="n">
-        <v>32.65</v>
+        <v>32.79</v>
       </c>
       <c r="I15" s="11" t="n">
-        <v>23.06</v>
+        <v>23.15</v>
       </c>
       <c r="J15" s="11" t="n">
         <v>10.44</v>
@@ -8250,7 +8250,7 @@
         <v>1.78</v>
       </c>
       <c r="N15" s="9" t="n">
-        <v>18.16</v>
+        <v>18.15</v>
       </c>
       <c r="O15" s="10" t="n">
         <v>-31.96</v>
@@ -8265,19 +8265,19 @@
         <v>66.5</v>
       </c>
       <c r="S15" s="17" t="n">
-        <v>65.90000000000001</v>
+        <v>65.7</v>
       </c>
       <c r="T15" s="11" t="n">
-        <v>27.87</v>
+        <v>28.19</v>
       </c>
       <c r="U15" s="18" t="n">
-        <v>0.586</v>
+        <v>0.585</v>
       </c>
       <c r="V15" s="18" t="n">
-        <v>0.185</v>
+        <v>0.184</v>
       </c>
       <c r="W15" s="11" t="n">
-        <v>1.28</v>
+        <v>1.3</v>
       </c>
       <c r="X15" s="17" t="n">
         <v>70</v>
@@ -8286,7 +8286,7 @@
         <v>13.7</v>
       </c>
       <c r="Z15" s="7" t="n">
-        <v>43.599</v>
+        <v>43.713</v>
       </c>
     </row>
     <row r="16">
@@ -8299,25 +8299,25 @@
         </is>
       </c>
       <c r="C16" s="20" t="n">
-        <v>68.59999999999999</v>
+        <v>68.7</v>
       </c>
       <c r="D16" s="22" t="n">
-        <v>20.38</v>
+        <v>20.3</v>
       </c>
       <c r="E16" s="22" t="n">
-        <v>23.89</v>
+        <v>24.04</v>
       </c>
       <c r="F16" s="22" t="n">
-        <v>14.77</v>
+        <v>14.61</v>
       </c>
       <c r="G16" s="22" t="n">
-        <v>9.800000000000001</v>
+        <v>9.84</v>
       </c>
       <c r="H16" s="22" t="n">
-        <v>20.46</v>
+        <v>20.69</v>
       </c>
       <c r="I16" s="22" t="n">
-        <v>19.57</v>
+        <v>19.69</v>
       </c>
       <c r="J16" s="22" t="n">
         <v>9.640000000000001</v>
@@ -8326,40 +8326,40 @@
         <v>8.35</v>
       </c>
       <c r="L16" s="23" t="n">
-        <v>1.38</v>
+        <v>1.39</v>
       </c>
       <c r="M16" s="23" t="n">
-        <v>1.96</v>
+        <v>1.97</v>
       </c>
       <c r="N16" s="23" t="n">
-        <v>15.65</v>
+        <v>15.64</v>
       </c>
       <c r="O16" s="21" t="n">
         <v>-39.06</v>
       </c>
       <c r="P16" s="23" t="n">
-        <v>0.61</v>
+        <v>0.62</v>
       </c>
       <c r="Q16" s="23" t="n">
-        <v>-1.41</v>
+        <v>-1.4</v>
       </c>
       <c r="R16" s="24" t="n">
         <v>19.1</v>
       </c>
       <c r="S16" s="24" t="n">
-        <v>5.2</v>
+        <v>4.8</v>
       </c>
       <c r="T16" s="22" t="n">
-        <v>27.27</v>
+        <v>27.44</v>
       </c>
       <c r="U16" s="25" t="n">
-        <v>0.117</v>
+        <v>0.116</v>
       </c>
       <c r="V16" s="25" t="n">
         <v>0.01</v>
       </c>
       <c r="W16" s="22" t="n">
-        <v>0.98</v>
+        <v>1.01</v>
       </c>
       <c r="X16" s="24" t="n">
         <v>72.2</v>
@@ -8368,7 +8368,7 @@
         <v>12</v>
       </c>
       <c r="Z16" s="19" t="n">
-        <v>47.2266</v>
+        <v>47.3982</v>
       </c>
     </row>
     <row r="17">
@@ -8381,25 +8381,25 @@
         </is>
       </c>
       <c r="C17" s="16" t="n">
-        <v>68.5</v>
+        <v>68.59999999999999</v>
       </c>
       <c r="D17" s="11" t="n">
-        <v>14.64</v>
+        <v>14.17</v>
       </c>
       <c r="E17" s="11" t="n">
-        <v>20.09</v>
+        <v>20.05</v>
       </c>
       <c r="F17" s="11" t="n">
-        <v>12.73</v>
+        <v>12.99</v>
       </c>
       <c r="G17" s="11" t="n">
-        <v>12.61</v>
+        <v>12.6</v>
       </c>
       <c r="H17" s="11" t="n">
-        <v>17.88</v>
+        <v>17.78</v>
       </c>
       <c r="I17" s="11" t="n">
-        <v>17.1</v>
+        <v>17.05</v>
       </c>
       <c r="J17" s="11" t="n">
         <v>10.35</v>
@@ -8408,13 +8408,13 @@
         <v>9.44</v>
       </c>
       <c r="L17" s="9" t="n">
-        <v>1.27</v>
+        <v>1.26</v>
       </c>
       <c r="M17" s="9" t="n">
         <v>1.71</v>
       </c>
       <c r="N17" s="9" t="n">
-        <v>13.26</v>
+        <v>13.25</v>
       </c>
       <c r="O17" s="10" t="n">
         <v>-30.06</v>
@@ -8432,7 +8432,7 @@
         <v>12.5</v>
       </c>
       <c r="T17" s="11" t="n">
-        <v>22.66</v>
+        <v>22.65</v>
       </c>
       <c r="U17" s="18" t="n">
         <v>0.155</v>
@@ -8441,7 +8441,7 @@
         <v>0.024</v>
       </c>
       <c r="W17" s="11" t="n">
-        <v>1.01</v>
+        <v>1.03</v>
       </c>
       <c r="X17" s="17" t="n">
         <v>73.2</v>
@@ -8450,7 +8450,7 @@
         <v>13.7</v>
       </c>
       <c r="Z17" s="7" t="n">
-        <v>47.5098</v>
+        <v>47.4644</v>
       </c>
     </row>
     <row r="18">
@@ -8466,22 +8466,22 @@
         <v>68.09999999999999</v>
       </c>
       <c r="D18" s="22" t="n">
-        <v>13.73</v>
+        <v>12.59</v>
       </c>
       <c r="E18" s="22" t="n">
-        <v>20.93</v>
+        <v>20.88</v>
       </c>
       <c r="F18" s="22" t="n">
-        <v>10.59</v>
+        <v>10.72</v>
       </c>
       <c r="G18" s="22" t="n">
-        <v>8.640000000000001</v>
+        <v>8.619999999999999</v>
       </c>
       <c r="H18" s="22" t="n">
-        <v>20.13</v>
+        <v>20.01</v>
       </c>
       <c r="I18" s="22" t="n">
-        <v>16.71</v>
+        <v>16.65</v>
       </c>
       <c r="J18" s="22" t="n">
         <v>13.03</v>
@@ -8490,13 +8490,13 @@
         <v>8.92</v>
       </c>
       <c r="L18" s="23" t="n">
-        <v>1.3</v>
+        <v>1.29</v>
       </c>
       <c r="M18" s="23" t="n">
         <v>1.69</v>
       </c>
       <c r="N18" s="23" t="n">
-        <v>14.34</v>
+        <v>14.33</v>
       </c>
       <c r="O18" s="21" t="n">
         <v>-27.06</v>
@@ -8514,7 +8514,7 @@
         <v>38.4</v>
       </c>
       <c r="T18" s="22" t="n">
-        <v>22.66</v>
+        <v>22.71</v>
       </c>
       <c r="U18" s="25" t="n">
         <v>0.362</v>
@@ -8523,7 +8523,7 @@
         <v>0.11</v>
       </c>
       <c r="W18" s="22" t="n">
-        <v>1.06</v>
+        <v>1.08</v>
       </c>
       <c r="X18" s="24" t="n">
         <v>79.8</v>
@@ -8532,7 +8532,7 @@
         <v>7</v>
       </c>
       <c r="Z18" s="19" t="n">
-        <v>22.9219</v>
+        <v>22.8945</v>
       </c>
     </row>
     <row r="19">
@@ -8627,25 +8627,25 @@
         </is>
       </c>
       <c r="C20" s="20" t="n">
-        <v>66.5</v>
+        <v>66.7</v>
       </c>
       <c r="D20" s="22" t="n">
-        <v>18.07</v>
+        <v>18.98</v>
       </c>
       <c r="E20" s="22" t="n">
-        <v>21.91</v>
+        <v>22.26</v>
       </c>
       <c r="F20" s="22" t="n">
-        <v>11.13</v>
+        <v>11.04</v>
       </c>
       <c r="G20" s="22" t="n">
-        <v>11.41</v>
+        <v>11.5</v>
       </c>
       <c r="H20" s="22" t="n">
-        <v>18.86</v>
+        <v>19.43</v>
       </c>
       <c r="I20" s="22" t="n">
-        <v>16.04</v>
+        <v>16.36</v>
       </c>
       <c r="J20" s="22" t="n">
         <v>10.65</v>
@@ -8654,19 +8654,19 @@
         <v>10.21</v>
       </c>
       <c r="L20" s="23" t="n">
-        <v>1.09</v>
+        <v>1.11</v>
       </c>
       <c r="M20" s="23" t="n">
-        <v>1.5</v>
+        <v>1.53</v>
       </c>
       <c r="N20" s="23" t="n">
-        <v>18.27</v>
+        <v>18.26</v>
       </c>
       <c r="O20" s="21" t="n">
         <v>-33.55</v>
       </c>
       <c r="P20" s="23" t="n">
-        <v>0.65</v>
+        <v>0.66</v>
       </c>
       <c r="Q20" s="23" t="n">
         <v>-1.8</v>
@@ -8675,19 +8675,19 @@
         <v>21.6</v>
       </c>
       <c r="S20" s="24" t="n">
-        <v>14.9</v>
+        <v>14.1</v>
       </c>
       <c r="T20" s="22" t="n">
-        <v>25.32</v>
+        <v>25.74</v>
       </c>
       <c r="U20" s="25" t="n">
-        <v>0.157</v>
+        <v>0.155</v>
       </c>
       <c r="V20" s="25" t="n">
         <v>0.013</v>
       </c>
       <c r="W20" s="22" t="n">
-        <v>0.84</v>
+        <v>0.87</v>
       </c>
       <c r="X20" s="24" t="n">
         <v>74</v>
@@ -8696,7 +8696,7 @@
         <v>12</v>
       </c>
       <c r="Z20" s="19" t="n">
-        <v>35.2769</v>
+        <v>35.5769</v>
       </c>
     </row>
     <row r="21">
@@ -9606,67 +9606,67 @@
           <t>Kotak Quality Overseas Equity Active FOF - Direct Plan - Growth-</t>
         </is>
       </c>
-      <c r="C32" s="20" t="n">
-        <v>50.1</v>
+      <c r="C32" s="26" t="n">
+        <v>49.9</v>
       </c>
       <c r="D32" s="22" t="n">
-        <v>15.21</v>
+        <v>14.88</v>
       </c>
       <c r="E32" s="22" t="n">
-        <v>4.83</v>
+        <v>4.73</v>
       </c>
       <c r="F32" s="22" t="n">
-        <v>2.87</v>
+        <v>2.81</v>
       </c>
       <c r="G32" s="22" t="n">
-        <v>1.43</v>
+        <v>1.4</v>
       </c>
       <c r="H32" s="21" t="n"/>
       <c r="I32" s="21" t="n"/>
       <c r="J32" s="21" t="n"/>
       <c r="K32" s="21" t="n"/>
       <c r="L32" s="23" t="n">
-        <v>2.61</v>
+        <v>2.52</v>
       </c>
       <c r="M32" s="23" t="n">
-        <v>3.56</v>
+        <v>3.45</v>
       </c>
       <c r="N32" s="23" t="n">
-        <v>11.36</v>
+        <v>11.32</v>
       </c>
       <c r="O32" s="23" t="n">
         <v>-3.86</v>
       </c>
       <c r="P32" s="23" t="n">
-        <v>1.25</v>
+        <v>1.23</v>
       </c>
       <c r="Q32" s="23" t="n">
-        <v>-0.93</v>
+        <v>-0.92</v>
       </c>
       <c r="R32" s="24" t="n">
         <v>16.2</v>
       </c>
       <c r="S32" s="24" t="n">
-        <v>-25</v>
+        <v>-22.6</v>
       </c>
       <c r="T32" s="22" t="n">
-        <v>36.15</v>
+        <v>35.04</v>
       </c>
       <c r="U32" s="25" t="n">
-        <v>0.025</v>
+        <v>0.029</v>
       </c>
       <c r="V32" s="25" t="n">
         <v>0.001</v>
       </c>
       <c r="W32" s="22" t="n">
-        <v>1.79</v>
+        <v>1.86</v>
       </c>
       <c r="X32" s="24" t="n"/>
       <c r="Y32" s="24" t="n">
         <v>0.5</v>
       </c>
       <c r="Z32" s="19" t="n">
-        <v>11.536</v>
+        <v>11.503</v>
       </c>
     </row>
     <row r="33">
@@ -32803,28 +32803,28 @@
         <v>6.5</v>
       </c>
       <c r="E79" s="11" t="n">
-        <v>6.96</v>
+        <v>6.95</v>
       </c>
       <c r="F79" s="11" t="n">
-        <v>4.46</v>
+        <v>4.47</v>
       </c>
       <c r="G79" s="11" t="n">
-        <v>2.2</v>
+        <v>2.21</v>
       </c>
       <c r="H79" s="11" t="n">
         <v>6.74</v>
       </c>
       <c r="I79" s="11" t="n">
-        <v>6.78</v>
+        <v>6.77</v>
       </c>
       <c r="J79" s="11" t="n">
+        <v>6.99</v>
+      </c>
+      <c r="K79" s="11" t="n">
         <v>7</v>
       </c>
-      <c r="K79" s="11" t="n">
-        <v>7.01</v>
-      </c>
       <c r="L79" s="9" t="n">
-        <v>-14.54</v>
+        <v>-14.56</v>
       </c>
       <c r="M79" s="9" t="n"/>
       <c r="N79" s="9" t="n">
@@ -32834,7 +32834,7 @@
         <v>-0.01</v>
       </c>
       <c r="P79" s="9" t="n">
-        <v>696</v>
+        <v>695</v>
       </c>
       <c r="Q79" s="9" t="n">
         <v>0.01</v>
@@ -32855,7 +32855,7 @@
         <v>0.006</v>
       </c>
       <c r="W79" s="10" t="n">
-        <v>-0.11</v>
+        <v>-0.12</v>
       </c>
       <c r="X79" s="17" t="n">
         <v>100</v>
@@ -32864,7 +32864,7 @@
         <v>3.2</v>
       </c>
       <c r="Z79" s="7" t="n">
-        <v>1243.8732</v>
+        <v>1244.469</v>
       </c>
     </row>
     <row r="80">
@@ -33793,19 +33793,19 @@
         </is>
       </c>
       <c r="C92" s="26" t="n">
-        <v>37</v>
+        <v>36.9</v>
       </c>
       <c r="D92" s="22" t="n">
-        <v>5.32</v>
+        <v>5.33</v>
       </c>
       <c r="E92" s="22" t="n">
         <v>6.07</v>
       </c>
       <c r="F92" s="22" t="n">
-        <v>3.93</v>
+        <v>3.94</v>
       </c>
       <c r="G92" s="22" t="n">
-        <v>1.94</v>
+        <v>1.95</v>
       </c>
       <c r="H92" s="22" t="n">
         <v>5.73</v>
@@ -33814,13 +33814,13 @@
         <v>5.79</v>
       </c>
       <c r="J92" s="22" t="n">
-        <v>6.2</v>
+        <v>6.19</v>
       </c>
       <c r="K92" s="22" t="n">
         <v>6.15</v>
       </c>
       <c r="L92" s="23" t="n">
-        <v>-40.06</v>
+        <v>-40.05</v>
       </c>
       <c r="M92" s="23" t="n"/>
       <c r="N92" s="23" t="n">
@@ -33849,7 +33849,7 @@
         <v>0.001</v>
       </c>
       <c r="W92" s="21" t="n">
-        <v>-0.16</v>
+        <v>-0.18</v>
       </c>
       <c r="X92" s="24" t="n">
         <v>100</v>
@@ -33858,7 +33858,7 @@
         <v>3.2</v>
       </c>
       <c r="Z92" s="19" t="n">
-        <v>1212.5268</v>
+        <v>1213.1952</v>
       </c>
     </row>
     <row r="93">
@@ -35648,38 +35648,38 @@
         </is>
       </c>
       <c r="C16" s="26" t="n">
-        <v>25.7</v>
+        <v>26.4</v>
       </c>
       <c r="D16" s="21" t="n">
-        <v>-8.19</v>
+        <v>-7.99</v>
       </c>
       <c r="E16" s="22" t="n">
-        <v>0.73</v>
+        <v>0.99</v>
       </c>
       <c r="F16" s="22" t="n">
-        <v>0.44</v>
+        <v>0.59</v>
       </c>
       <c r="G16" s="22" t="n">
-        <v>0.22</v>
+        <v>0.3</v>
       </c>
       <c r="H16" s="21" t="n">
-        <v>-6.2</v>
+        <v>-5.63</v>
       </c>
       <c r="I16" s="21" t="n">
-        <v>-6.2</v>
+        <v>-5.63</v>
       </c>
       <c r="J16" s="21" t="n">
-        <v>-3.34</v>
+        <v>-3.33</v>
       </c>
       <c r="K16" s="21" t="n"/>
       <c r="L16" s="23" t="n">
-        <v>-0.25</v>
+        <v>-0.23</v>
       </c>
       <c r="M16" s="23" t="n">
-        <v>-0.37</v>
+        <v>-0.34</v>
       </c>
       <c r="N16" s="23" t="n">
-        <v>16.97</v>
+        <v>16.96</v>
       </c>
       <c r="O16" s="21" t="n">
         <v>-28.59</v>
@@ -35694,19 +35694,19 @@
         <v>81.3</v>
       </c>
       <c r="S16" s="24" t="n">
-        <v>94.8</v>
+        <v>94.40000000000001</v>
       </c>
       <c r="T16" s="22" t="n">
-        <v>0.63</v>
+        <v>1.25</v>
       </c>
       <c r="U16" s="25" t="n">
-        <v>0.856</v>
+        <v>0.853</v>
       </c>
       <c r="V16" s="25" t="n">
-        <v>0.468</v>
+        <v>0.465</v>
       </c>
       <c r="W16" s="22" t="n">
-        <v>0.03</v>
+        <v>0.08</v>
       </c>
       <c r="X16" s="24" t="n">
         <v>25.6</v>
@@ -35715,7 +35715,7 @@
         <v>2.6</v>
       </c>
       <c r="Z16" s="19" t="n">
-        <v>10.24</v>
+        <v>10.319</v>
       </c>
     </row>
   </sheetData>
@@ -41992,25 +41992,25 @@
         </is>
       </c>
       <c r="C4" s="20" t="n">
-        <v>65.8</v>
+        <v>65.3</v>
       </c>
       <c r="D4" s="21" t="n">
-        <v>-0.73</v>
+        <v>-1.92</v>
       </c>
       <c r="E4" s="22" t="n">
-        <v>12.78</v>
+        <v>12.6</v>
       </c>
       <c r="F4" s="22" t="n">
-        <v>12.59</v>
+        <v>12.3</v>
       </c>
       <c r="G4" s="22" t="n">
-        <v>14.9</v>
+        <v>14.85</v>
       </c>
       <c r="H4" s="22" t="n">
-        <v>5.53</v>
+        <v>5.21</v>
       </c>
       <c r="I4" s="22" t="n">
-        <v>11.58</v>
+        <v>11.37</v>
       </c>
       <c r="J4" s="22" t="n">
         <v>17.91</v>
@@ -42019,10 +42019,10 @@
         <v>17.24</v>
       </c>
       <c r="L4" s="23" t="n">
-        <v>0.73</v>
+        <v>0.71</v>
       </c>
       <c r="M4" s="23" t="n">
-        <v>0.99</v>
+        <v>0.97</v>
       </c>
       <c r="N4" s="23" t="n">
         <v>10.23</v>
@@ -42031,7 +42031,7 @@
         <v>-35.74</v>
       </c>
       <c r="P4" s="23" t="n">
-        <v>0.36</v>
+        <v>0.35</v>
       </c>
       <c r="Q4" s="23" t="n">
         <v>-1.07</v>
@@ -42043,7 +42043,7 @@
         <v>79.8</v>
       </c>
       <c r="T4" s="22" t="n">
-        <v>9.33</v>
+        <v>9.380000000000001</v>
       </c>
       <c r="U4" s="25" t="n">
         <v>0.702</v>
@@ -42052,7 +42052,7 @@
         <v>0.789</v>
       </c>
       <c r="W4" s="22" t="n">
-        <v>1.17</v>
+        <v>1.2</v>
       </c>
       <c r="X4" s="24" t="n">
         <v>90</v>
@@ -42061,7 +42061,7 @@
         <v>13.5</v>
       </c>
       <c r="Z4" s="19" t="n">
-        <v>236.2361</v>
+        <v>235.1588</v>
       </c>
     </row>
     <row r="5">
@@ -44957,7 +44957,7 @@
     </row>
     <row r="7">
       <c r="A7" s="7" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="B7" s="7" t="inlineStr">
         <is>
@@ -44965,25 +44965,25 @@
         </is>
       </c>
       <c r="C7" s="16" t="n">
-        <v>59.5</v>
+        <v>59</v>
       </c>
       <c r="D7" s="11" t="n">
-        <v>1.26</v>
+        <v>0.23</v>
       </c>
       <c r="E7" s="11" t="n">
-        <v>10.2</v>
+        <v>10</v>
       </c>
       <c r="F7" s="11" t="n">
-        <v>10.4</v>
+        <v>10.21</v>
       </c>
       <c r="G7" s="11" t="n">
-        <v>11.85</v>
+        <v>11.79</v>
       </c>
       <c r="H7" s="11" t="n">
-        <v>5.53</v>
+        <v>5.16</v>
       </c>
       <c r="I7" s="11" t="n">
-        <v>9.359999999999999</v>
+        <v>9.130000000000001</v>
       </c>
       <c r="J7" s="11" t="n">
         <v>13.46</v>
@@ -44992,19 +44992,19 @@
         <v>13.14</v>
       </c>
       <c r="L7" s="9" t="n">
-        <v>0.71</v>
+        <v>0.67</v>
       </c>
       <c r="M7" s="9" t="n">
-        <v>0.9399999999999999</v>
+        <v>0.9</v>
       </c>
       <c r="N7" s="9" t="n">
-        <v>6.32</v>
+        <v>6.33</v>
       </c>
       <c r="O7" s="10" t="n">
         <v>-26.35</v>
       </c>
       <c r="P7" s="9" t="n">
-        <v>0.39</v>
+        <v>0.38</v>
       </c>
       <c r="Q7" s="9" t="n">
         <v>-0.58</v>
@@ -45013,10 +45013,10 @@
         <v>30.7</v>
       </c>
       <c r="S7" s="17" t="n">
-        <v>55.5</v>
+        <v>55.7</v>
       </c>
       <c r="T7" s="11" t="n">
-        <v>7.96</v>
+        <v>7.88</v>
       </c>
       <c r="U7" s="18" t="n">
         <v>0.426</v>
@@ -45025,16 +45025,16 @@
         <v>0.759</v>
       </c>
       <c r="W7" s="11" t="n">
-        <v>0.49</v>
+        <v>0.51</v>
       </c>
       <c r="X7" s="17" t="n">
-        <v>96.40000000000001</v>
+        <v>96.2</v>
       </c>
       <c r="Y7" s="17" t="n">
         <v>13.7</v>
       </c>
       <c r="Z7" s="7" t="n">
-        <v>135.2014</v>
+        <v>134.4748</v>
       </c>
     </row>
     <row r="8">
@@ -51297,31 +51297,31 @@
         <v>6.54</v>
       </c>
       <c r="E3" s="11" t="n">
-        <v>7</v>
+        <v>6.99</v>
       </c>
       <c r="F3" s="11" t="n">
-        <v>6.41</v>
+        <v>6.42</v>
       </c>
       <c r="G3" s="11" t="n">
-        <v>68.09999999999999</v>
+        <v>68.11</v>
       </c>
       <c r="H3" s="11" t="n">
-        <v>6.79</v>
+        <v>6.78</v>
       </c>
       <c r="I3" s="11" t="n">
         <v>6.81</v>
       </c>
       <c r="J3" s="11" t="n">
-        <v>717.15</v>
+        <v>715.61</v>
       </c>
       <c r="K3" s="11" t="n">
-        <v>39.66</v>
+        <v>39.56</v>
       </c>
       <c r="L3" s="9" t="n">
-        <v>-13.29</v>
+        <v>-13.31</v>
       </c>
       <c r="M3" s="9" t="n">
-        <v>-30.17</v>
+        <v>-30.2</v>
       </c>
       <c r="N3" s="9" t="n">
         <v>0.13</v>
@@ -51330,7 +51330,7 @@
         <v>-0.15</v>
       </c>
       <c r="P3" s="9" t="n">
-        <v>46.67</v>
+        <v>46.6</v>
       </c>
       <c r="Q3" s="9" t="n">
         <v>0.01</v>
@@ -51348,19 +51348,19 @@
         <v>0.001</v>
       </c>
       <c r="V3" s="18" t="n">
-        <v>0.007</v>
+        <v>0.008</v>
       </c>
       <c r="W3" s="10" t="n">
-        <v>-0.11</v>
+        <v>-0.12</v>
       </c>
       <c r="X3" s="17" t="n">
         <v>100</v>
       </c>
       <c r="Y3" s="17" t="n">
-        <v>9.800000000000001</v>
+        <v>9.9</v>
       </c>
       <c r="Z3" s="7" t="n">
-        <v>3684.5801</v>
+        <v>3686.4082</v>
       </c>
     </row>
     <row r="4">
@@ -51459,7 +51459,7 @@
         <v>6.49</v>
       </c>
       <c r="E5" s="11" t="n">
-        <v>6.96</v>
+        <v>6.95</v>
       </c>
       <c r="F5" s="11" t="n">
         <v>6.38</v>
@@ -51468,19 +51468,19 @@
         <v>6.13</v>
       </c>
       <c r="H5" s="11" t="n">
-        <v>6.75</v>
+        <v>6.74</v>
       </c>
       <c r="I5" s="11" t="n">
         <v>6.77</v>
       </c>
       <c r="J5" s="11" t="n">
-        <v>854.4</v>
+        <v>853.13</v>
       </c>
       <c r="K5" s="11" t="n">
-        <v>46.79</v>
+        <v>46.72</v>
       </c>
       <c r="L5" s="9" t="n">
-        <v>-13.95</v>
+        <v>-13.97</v>
       </c>
       <c r="M5" s="9" t="n"/>
       <c r="N5" s="9" t="n">
@@ -51490,7 +51490,7 @@
         <v>-0.23</v>
       </c>
       <c r="P5" s="9" t="n">
-        <v>30.26</v>
+        <v>30.22</v>
       </c>
       <c r="Q5" s="9" t="n">
         <v>0.01</v>
@@ -51511,16 +51511,16 @@
         <v>0.007</v>
       </c>
       <c r="W5" s="10" t="n">
-        <v>-0.11</v>
+        <v>-0.12</v>
       </c>
       <c r="X5" s="17" t="n">
         <v>100</v>
       </c>
       <c r="Y5" s="17" t="n">
-        <v>13.7</v>
+        <v>13.8</v>
       </c>
       <c r="Z5" s="7" t="n">
-        <v>4498.0774</v>
+        <v>4500.3095</v>
       </c>
     </row>
     <row r="6">
@@ -51539,31 +51539,31 @@
         <v>6.48</v>
       </c>
       <c r="E6" s="22" t="n">
-        <v>6.92</v>
+        <v>6.91</v>
       </c>
       <c r="F6" s="22" t="n">
-        <v>6.35</v>
+        <v>6.36</v>
       </c>
       <c r="G6" s="22" t="n">
         <v>6.06</v>
       </c>
       <c r="H6" s="22" t="n">
-        <v>6.72</v>
+        <v>6.71</v>
       </c>
       <c r="I6" s="22" t="n">
         <v>6.74</v>
       </c>
       <c r="J6" s="22" t="n">
-        <v>845.15</v>
+        <v>843.89</v>
       </c>
       <c r="K6" s="22" t="n">
-        <v>104.02</v>
+        <v>103.85</v>
       </c>
       <c r="L6" s="23" t="n">
-        <v>-13.04</v>
+        <v>-13.06</v>
       </c>
       <c r="M6" s="23" t="n">
-        <v>-29.47</v>
+        <v>-29.51</v>
       </c>
       <c r="N6" s="23" t="n">
         <v>0.13</v>
@@ -51572,7 +51572,7 @@
         <v>-0.18</v>
       </c>
       <c r="P6" s="23" t="n">
-        <v>38.44</v>
+        <v>38.39</v>
       </c>
       <c r="Q6" s="23" t="n">
         <v>0.01</v>
@@ -51593,16 +51593,16 @@
         <v>0.005</v>
       </c>
       <c r="W6" s="21" t="n">
-        <v>-0.11</v>
+        <v>-0.13</v>
       </c>
       <c r="X6" s="24" t="n">
         <v>100</v>
       </c>
       <c r="Y6" s="24" t="n">
-        <v>13.7</v>
+        <v>13.8</v>
       </c>
       <c r="Z6" s="19" t="n">
-        <v>5595.3756</v>
+        <v>5598.0849</v>
       </c>
     </row>
     <row r="7">
@@ -51624,25 +51624,25 @@
         <v>6.93</v>
       </c>
       <c r="F7" s="11" t="n">
-        <v>6.36</v>
+        <v>6.37</v>
       </c>
       <c r="G7" s="11" t="n">
-        <v>6.08</v>
+        <v>6.07</v>
       </c>
       <c r="H7" s="11" t="n">
-        <v>6.74</v>
+        <v>6.73</v>
       </c>
       <c r="I7" s="11" t="n">
         <v>6.76</v>
       </c>
       <c r="J7" s="11" t="n">
-        <v>55.53</v>
+        <v>55.45</v>
       </c>
       <c r="K7" s="11" t="n">
         <v>8.6</v>
       </c>
       <c r="L7" s="9" t="n">
-        <v>-9.35</v>
+        <v>-9.359999999999999</v>
       </c>
       <c r="M7" s="9" t="n"/>
       <c r="N7" s="9" t="n">
@@ -51673,16 +51673,16 @@
         <v>0.006</v>
       </c>
       <c r="W7" s="10" t="n">
-        <v>-0.11</v>
+        <v>-0.12</v>
       </c>
       <c r="X7" s="17" t="n">
         <v>100</v>
       </c>
       <c r="Y7" s="17" t="n">
-        <v>13.7</v>
+        <v>13.8</v>
       </c>
       <c r="Z7" s="7" t="n">
-        <v>5757.3659</v>
+        <v>5760.2029</v>
       </c>
     </row>
     <row r="8">
@@ -51701,7 +51701,7 @@
         <v>6.48</v>
       </c>
       <c r="E8" s="22" t="n">
-        <v>6.93</v>
+        <v>6.92</v>
       </c>
       <c r="F8" s="22" t="n">
         <v>6.36</v>
@@ -51710,19 +51710,19 @@
         <v>6.13</v>
       </c>
       <c r="H8" s="22" t="n">
-        <v>6.72</v>
+        <v>6.71</v>
       </c>
       <c r="I8" s="22" t="n">
         <v>6.75</v>
       </c>
       <c r="J8" s="22" t="n">
-        <v>55.53</v>
+        <v>55.45</v>
       </c>
       <c r="K8" s="22" t="n">
         <v>8.65</v>
       </c>
       <c r="L8" s="23" t="n">
-        <v>-13.66</v>
+        <v>-13.68</v>
       </c>
       <c r="M8" s="23" t="n"/>
       <c r="N8" s="23" t="n">
@@ -51732,7 +51732,7 @@
         <v>-0.16</v>
       </c>
       <c r="P8" s="23" t="n">
-        <v>43.31</v>
+        <v>43.25</v>
       </c>
       <c r="Q8" s="23" t="n">
         <v>0.01</v>
@@ -51744,25 +51744,25 @@
         <v>-6</v>
       </c>
       <c r="T8" s="22" t="n">
-        <v>4.81</v>
+        <v>4.8</v>
       </c>
       <c r="U8" s="25" t="n">
         <v>0.001</v>
       </c>
       <c r="V8" s="25" t="n">
-        <v>0.005</v>
+        <v>0.006</v>
       </c>
       <c r="W8" s="21" t="n">
-        <v>-0.11</v>
+        <v>-0.13</v>
       </c>
       <c r="X8" s="24" t="n">
         <v>100</v>
       </c>
       <c r="Y8" s="24" t="n">
-        <v>13.7</v>
+        <v>13.8</v>
       </c>
       <c r="Z8" s="19" t="n">
-        <v>5172.632</v>
+        <v>5175.1681</v>
       </c>
     </row>
     <row r="9">
@@ -52258,7 +52258,7 @@
         <v>6.99</v>
       </c>
       <c r="F15" s="11" t="n">
-        <v>6.42</v>
+        <v>6.43</v>
       </c>
       <c r="G15" s="11" t="n">
         <v>6.16</v>
@@ -52276,7 +52276,7 @@
         <v>6.55</v>
       </c>
       <c r="L15" s="9" t="n">
-        <v>-13.2</v>
+        <v>-13.22</v>
       </c>
       <c r="M15" s="9" t="n"/>
       <c r="N15" s="9" t="n">
@@ -52307,16 +52307,16 @@
         <v>0.006</v>
       </c>
       <c r="W15" s="10" t="n">
-        <v>-0.11</v>
+        <v>-0.12</v>
       </c>
       <c r="X15" s="17" t="n">
         <v>100</v>
       </c>
       <c r="Y15" s="17" t="n">
-        <v>13.7</v>
+        <v>13.8</v>
       </c>
       <c r="Z15" s="7" t="n">
-        <v>3171.4023</v>
+        <v>3172.9339</v>
       </c>
     </row>
     <row r="16">
@@ -52335,13 +52335,13 @@
         <v>6.57</v>
       </c>
       <c r="E16" s="22" t="n">
-        <v>7</v>
+        <v>6.99</v>
       </c>
       <c r="F16" s="22" t="n">
         <v>6.44</v>
       </c>
       <c r="G16" s="22" t="n">
-        <v>6.18</v>
+        <v>6.17</v>
       </c>
       <c r="H16" s="22" t="n">
         <v>6.8</v>
@@ -52356,7 +52356,7 @@
         <v>6.58</v>
       </c>
       <c r="L16" s="23" t="n">
-        <v>-13.07</v>
+        <v>-13.09</v>
       </c>
       <c r="M16" s="23" t="n"/>
       <c r="N16" s="23" t="n">
@@ -52366,7 +52366,7 @@
         <v>-0.23</v>
       </c>
       <c r="P16" s="23" t="n">
-        <v>30.43</v>
+        <v>30.39</v>
       </c>
       <c r="Q16" s="23" t="n">
         <v>0.01</v>
@@ -52387,16 +52387,16 @@
         <v>0.005</v>
       </c>
       <c r="W16" s="21" t="n">
-        <v>-0.11</v>
+        <v>-0.12</v>
       </c>
       <c r="X16" s="24" t="n">
         <v>100</v>
       </c>
       <c r="Y16" s="24" t="n">
-        <v>13.7</v>
+        <v>13.8</v>
       </c>
       <c r="Z16" s="19" t="n">
-        <v>460.5501</v>
+        <v>460.7809</v>
       </c>
     </row>
     <row r="17">
@@ -52415,19 +52415,19 @@
         <v>6.53</v>
       </c>
       <c r="E17" s="11" t="n">
-        <v>6.98</v>
+        <v>6.97</v>
       </c>
       <c r="F17" s="11" t="n">
-        <v>6.39</v>
+        <v>6.4</v>
       </c>
       <c r="G17" s="11" t="n">
         <v>6.17</v>
       </c>
       <c r="H17" s="11" t="n">
+        <v>6.78</v>
+      </c>
+      <c r="I17" s="11" t="n">
         <v>6.79</v>
-      </c>
-      <c r="I17" s="11" t="n">
-        <v>6.8</v>
       </c>
       <c r="J17" s="11" t="n">
         <v>6.83</v>
@@ -52436,7 +52436,7 @@
         <v>6.59</v>
       </c>
       <c r="L17" s="9" t="n">
-        <v>-13.47</v>
+        <v>-13.49</v>
       </c>
       <c r="M17" s="9" t="n"/>
       <c r="N17" s="9" t="n">
@@ -52446,7 +52446,7 @@
         <v>-0.16</v>
       </c>
       <c r="P17" s="9" t="n">
-        <v>43.62</v>
+        <v>43.56</v>
       </c>
       <c r="Q17" s="9" t="n">
         <v>0.01</v>
@@ -52467,66 +52467,66 @@
         <v>0.007</v>
       </c>
       <c r="W17" s="10" t="n">
-        <v>-0.11</v>
+        <v>-0.12</v>
       </c>
       <c r="X17" s="17" t="n">
         <v>100</v>
       </c>
       <c r="Y17" s="17" t="n">
-        <v>13.7</v>
+        <v>13.8</v>
       </c>
       <c r="Z17" s="7" t="n">
-        <v>4285.0759</v>
+        <v>4287.1191</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="19" t="n">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="B18" s="19" t="inlineStr">
         <is>
-          <t>Nippon India Liquid Fund - Direct Plan Growth Plan - Growth Option</t>
+          <t>BANK OF INDIA Liquid Fund- Direct Plan- Growth</t>
         </is>
       </c>
       <c r="C18" s="26" t="n">
-        <v>46.7</v>
+        <v>46.6</v>
       </c>
       <c r="D18" s="22" t="n">
-        <v>6.54</v>
+        <v>6.51</v>
       </c>
       <c r="E18" s="22" t="n">
-        <v>6.97</v>
+        <v>6.96</v>
       </c>
       <c r="F18" s="22" t="n">
-        <v>6.4</v>
+        <v>6.41</v>
       </c>
       <c r="G18" s="22" t="n">
-        <v>6.16</v>
+        <v>6.11</v>
       </c>
       <c r="H18" s="22" t="n">
-        <v>6.77</v>
+        <v>6.75</v>
       </c>
       <c r="I18" s="22" t="n">
-        <v>6.8</v>
+        <v>6.79</v>
       </c>
       <c r="J18" s="22" t="n">
-        <v>6.79</v>
+        <v>6.76</v>
       </c>
       <c r="K18" s="22" t="n">
-        <v>6.56</v>
+        <v>6.52</v>
       </c>
       <c r="L18" s="23" t="n">
-        <v>-13.24</v>
+        <v>-14.27</v>
       </c>
       <c r="M18" s="23" t="n"/>
       <c r="N18" s="23" t="n">
-        <v>0.13</v>
+        <v>0.12</v>
       </c>
       <c r="O18" s="23" t="n">
-        <v>-0.24</v>
+        <v>-0.16</v>
       </c>
       <c r="P18" s="23" t="n">
-        <v>29.04</v>
+        <v>43.5</v>
       </c>
       <c r="Q18" s="23" t="n">
         <v>0.01</v>
@@ -52538,75 +52538,75 @@
         <v>-6.1</v>
       </c>
       <c r="T18" s="22" t="n">
-        <v>4.85</v>
+        <v>4.82</v>
       </c>
       <c r="U18" s="25" t="n">
         <v>0.001</v>
       </c>
       <c r="V18" s="25" t="n">
-        <v>0.006</v>
+        <v>0.008</v>
       </c>
       <c r="W18" s="21" t="n">
-        <v>-0.11</v>
+        <v>-0.13</v>
       </c>
       <c r="X18" s="24" t="n">
         <v>100</v>
       </c>
       <c r="Y18" s="24" t="n">
-        <v>13.7</v>
+        <v>13.8</v>
       </c>
       <c r="Z18" s="19" t="n">
-        <v>6978.275</v>
+        <v>3284.12</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="7" t="n">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B19" s="7" t="inlineStr">
         <is>
-          <t>BANK OF INDIA Liquid Fund- Direct Plan- Growth</t>
+          <t>Nippon India Liquid Fund - Direct Plan Growth Plan - Growth Option</t>
         </is>
       </c>
       <c r="C19" s="27" t="n">
         <v>46.6</v>
       </c>
       <c r="D19" s="11" t="n">
-        <v>6.51</v>
+        <v>6.54</v>
       </c>
       <c r="E19" s="11" t="n">
-        <v>6.96</v>
+        <v>6.97</v>
       </c>
       <c r="F19" s="11" t="n">
         <v>6.41</v>
       </c>
       <c r="G19" s="11" t="n">
-        <v>6.11</v>
+        <v>6.16</v>
       </c>
       <c r="H19" s="11" t="n">
-        <v>6.75</v>
+        <v>6.77</v>
       </c>
       <c r="I19" s="11" t="n">
         <v>6.79</v>
       </c>
       <c r="J19" s="11" t="n">
-        <v>6.76</v>
+        <v>6.79</v>
       </c>
       <c r="K19" s="11" t="n">
-        <v>6.52</v>
+        <v>6.56</v>
       </c>
       <c r="L19" s="9" t="n">
-        <v>-14.27</v>
+        <v>-13.26</v>
       </c>
       <c r="M19" s="9" t="n"/>
       <c r="N19" s="9" t="n">
-        <v>0.12</v>
+        <v>0.13</v>
       </c>
       <c r="O19" s="9" t="n">
-        <v>-0.16</v>
+        <v>-0.24</v>
       </c>
       <c r="P19" s="9" t="n">
-        <v>43.5</v>
+        <v>29.04</v>
       </c>
       <c r="Q19" s="9" t="n">
         <v>0.01</v>
@@ -52618,30 +52618,30 @@
         <v>-6.1</v>
       </c>
       <c r="T19" s="11" t="n">
-        <v>4.82</v>
+        <v>4.85</v>
       </c>
       <c r="U19" s="18" t="n">
         <v>0.001</v>
       </c>
       <c r="V19" s="18" t="n">
-        <v>0.008</v>
+        <v>0.006</v>
       </c>
       <c r="W19" s="10" t="n">
-        <v>-0.13</v>
+        <v>-0.12</v>
       </c>
       <c r="X19" s="17" t="n">
         <v>100</v>
       </c>
       <c r="Y19" s="17" t="n">
-        <v>13.7</v>
+        <v>13.8</v>
       </c>
       <c r="Z19" s="7" t="n">
-        <v>3283.0326</v>
+        <v>6981.6712</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="19" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="B20" s="19" t="inlineStr">
         <is>
@@ -52649,13 +52649,13 @@
         </is>
       </c>
       <c r="C20" s="26" t="n">
-        <v>46.6</v>
+        <v>46.5</v>
       </c>
       <c r="D20" s="22" t="n">
-        <v>6.51</v>
+        <v>6.49</v>
       </c>
       <c r="E20" s="22" t="n">
-        <v>6.97</v>
+        <v>6.96</v>
       </c>
       <c r="F20" s="22" t="n">
         <v>6.29</v>
@@ -52676,7 +52676,7 @@
         <v>6.48</v>
       </c>
       <c r="L20" s="23" t="n">
-        <v>-6.14</v>
+        <v>-6.15</v>
       </c>
       <c r="M20" s="23" t="n"/>
       <c r="N20" s="23" t="n">
@@ -52686,7 +52686,7 @@
         <v>-0.25</v>
       </c>
       <c r="P20" s="23" t="n">
-        <v>27.88</v>
+        <v>27.84</v>
       </c>
       <c r="Q20" s="23" t="n">
         <v>0.01</v>
@@ -52707,66 +52707,68 @@
         <v>0.01</v>
       </c>
       <c r="W20" s="21" t="n">
-        <v>-0.11</v>
+        <v>-0.12</v>
       </c>
       <c r="X20" s="24" t="n">
         <v>100</v>
       </c>
       <c r="Y20" s="24" t="n">
-        <v>13.7</v>
+        <v>13.8</v>
       </c>
       <c r="Z20" s="19" t="n">
-        <v>2762.7293</v>
+        <v>2764.0743</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="7" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="B21" s="7" t="inlineStr">
         <is>
-          <t>Baroda BNP Paribas LIQUID FUND - DIRECT PLAN - GROWTH OPTION</t>
+          <t>BANDHAN LIQUID Fund -Direct Plan-Growth</t>
         </is>
       </c>
       <c r="C21" s="27" t="n">
-        <v>46.6</v>
+        <v>46.5</v>
       </c>
       <c r="D21" s="11" t="n">
-        <v>6.45</v>
+        <v>6.48</v>
       </c>
       <c r="E21" s="11" t="n">
-        <v>6.91</v>
+        <v>6.92</v>
       </c>
       <c r="F21" s="11" t="n">
-        <v>6.38</v>
+        <v>6.37</v>
       </c>
       <c r="G21" s="11" t="n">
-        <v>6.14</v>
+        <v>6.05</v>
       </c>
       <c r="H21" s="11" t="n">
-        <v>6.7</v>
+        <v>6.71</v>
       </c>
       <c r="I21" s="11" t="n">
         <v>6.75</v>
       </c>
       <c r="J21" s="11" t="n">
-        <v>6.8</v>
+        <v>6.7</v>
       </c>
       <c r="K21" s="11" t="n">
-        <v>6.57</v>
+        <v>6.46</v>
       </c>
       <c r="L21" s="9" t="n">
-        <v>-14.64</v>
-      </c>
-      <c r="M21" s="9" t="n"/>
+        <v>-13.83</v>
+      </c>
+      <c r="M21" s="9" t="n">
+        <v>-45.86</v>
+      </c>
       <c r="N21" s="9" t="n">
-        <v>0.12</v>
+        <v>0.13</v>
       </c>
       <c r="O21" s="9" t="n">
-        <v>-0.21</v>
+        <v>-0.23</v>
       </c>
       <c r="P21" s="9" t="n">
-        <v>32.9</v>
+        <v>30.09</v>
       </c>
       <c r="Q21" s="9" t="n">
         <v>0.01</v>
@@ -52775,78 +52777,78 @@
         <v>1.4</v>
       </c>
       <c r="S21" s="17" t="n">
-        <v>-6.1</v>
+        <v>-6</v>
       </c>
       <c r="T21" s="11" t="n">
-        <v>4.8</v>
+        <v>4.81</v>
       </c>
       <c r="U21" s="18" t="n">
         <v>0.001</v>
       </c>
       <c r="V21" s="18" t="n">
-        <v>0.005</v>
+        <v>0.006</v>
       </c>
       <c r="W21" s="10" t="n">
-        <v>-0.11</v>
+        <v>-0.13</v>
       </c>
       <c r="X21" s="17" t="n">
         <v>100</v>
       </c>
       <c r="Y21" s="17" t="n">
-        <v>13.7</v>
+        <v>13.8</v>
       </c>
       <c r="Z21" s="7" t="n">
-        <v>3283.8129</v>
+        <v>3442.33</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="19" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="B22" s="19" t="inlineStr">
         <is>
-          <t>HSBC Liquid Fund -  Growth Direct</t>
+          <t>Baroda BNP Paribas LIQUID FUND - DIRECT PLAN - GROWTH OPTION</t>
         </is>
       </c>
       <c r="C22" s="26" t="n">
-        <v>46.6</v>
+        <v>46.5</v>
       </c>
       <c r="D22" s="22" t="n">
-        <v>6.47</v>
+        <v>6.45</v>
       </c>
       <c r="E22" s="22" t="n">
-        <v>6.94</v>
+        <v>6.91</v>
       </c>
       <c r="F22" s="22" t="n">
         <v>6.39</v>
       </c>
       <c r="G22" s="22" t="n">
-        <v>6.11</v>
+        <v>6.14</v>
       </c>
       <c r="H22" s="22" t="n">
-        <v>6.73</v>
+        <v>6.69</v>
       </c>
       <c r="I22" s="22" t="n">
-        <v>6.77</v>
+        <v>6.75</v>
       </c>
       <c r="J22" s="22" t="n">
-        <v>6.75</v>
+        <v>6.8</v>
       </c>
       <c r="K22" s="22" t="n">
-        <v>6.51</v>
+        <v>6.57</v>
       </c>
       <c r="L22" s="23" t="n">
-        <v>-13.38</v>
+        <v>-14.66</v>
       </c>
       <c r="M22" s="23" t="n"/>
       <c r="N22" s="23" t="n">
-        <v>0.13</v>
+        <v>0.12</v>
       </c>
       <c r="O22" s="23" t="n">
-        <v>-0.27</v>
+        <v>-0.21</v>
       </c>
       <c r="P22" s="23" t="n">
-        <v>25.7</v>
+        <v>32.9</v>
       </c>
       <c r="Q22" s="23" t="n">
         <v>0.01</v>
@@ -52858,75 +52860,75 @@
         <v>-6.1</v>
       </c>
       <c r="T22" s="22" t="n">
-        <v>4.82</v>
+        <v>4.8</v>
       </c>
       <c r="U22" s="25" t="n">
         <v>0.001</v>
       </c>
       <c r="V22" s="25" t="n">
-        <v>0.007</v>
+        <v>0.005</v>
       </c>
       <c r="W22" s="21" t="n">
-        <v>-0.11</v>
+        <v>-0.13</v>
       </c>
       <c r="X22" s="24" t="n">
         <v>100</v>
       </c>
       <c r="Y22" s="24" t="n">
-        <v>13.7</v>
+        <v>13.8</v>
       </c>
       <c r="Z22" s="19" t="n">
-        <v>2839.1097</v>
+        <v>3285.4152</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="7" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="B23" s="7" t="inlineStr">
         <is>
-          <t>ICICI Prudential Liquid Fund - Direct Plan - Growth</t>
+          <t>HSBC Liquid Fund -  Growth Direct</t>
         </is>
       </c>
       <c r="C23" s="27" t="n">
-        <v>46.6</v>
+        <v>46.5</v>
       </c>
       <c r="D23" s="11" t="n">
-        <v>6.46</v>
+        <v>6.47</v>
       </c>
       <c r="E23" s="11" t="n">
-        <v>6.93</v>
+        <v>6.94</v>
       </c>
       <c r="F23" s="11" t="n">
-        <v>6.36</v>
+        <v>6.39</v>
       </c>
       <c r="G23" s="11" t="n">
         <v>6.11</v>
       </c>
       <c r="H23" s="11" t="n">
-        <v>6.72</v>
+        <v>6.73</v>
       </c>
       <c r="I23" s="11" t="n">
+        <v>6.77</v>
+      </c>
+      <c r="J23" s="11" t="n">
         <v>6.75</v>
       </c>
-      <c r="J23" s="11" t="n">
-        <v>6.76</v>
-      </c>
       <c r="K23" s="11" t="n">
-        <v>6.52</v>
+        <v>6.51</v>
       </c>
       <c r="L23" s="9" t="n">
-        <v>-13.7</v>
+        <v>-13.4</v>
       </c>
       <c r="M23" s="9" t="n"/>
       <c r="N23" s="9" t="n">
         <v>0.13</v>
       </c>
       <c r="O23" s="9" t="n">
-        <v>-0.16</v>
+        <v>-0.27</v>
       </c>
       <c r="P23" s="9" t="n">
-        <v>43.31</v>
+        <v>25.7</v>
       </c>
       <c r="Q23" s="9" t="n">
         <v>0.01</v>
@@ -52935,78 +52937,78 @@
         <v>1.4</v>
       </c>
       <c r="S23" s="17" t="n">
-        <v>-6.1</v>
+        <v>-6</v>
       </c>
       <c r="T23" s="11" t="n">
-        <v>4.83</v>
+        <v>4.81</v>
       </c>
       <c r="U23" s="18" t="n">
         <v>0.001</v>
       </c>
       <c r="V23" s="18" t="n">
-        <v>0.006</v>
+        <v>0.007</v>
       </c>
       <c r="W23" s="10" t="n">
-        <v>-0.11</v>
+        <v>-0.13</v>
       </c>
       <c r="X23" s="17" t="n">
         <v>100</v>
       </c>
       <c r="Y23" s="17" t="n">
-        <v>13.7</v>
+        <v>13.8</v>
       </c>
       <c r="Z23" s="7" t="n">
-        <v>421.6595</v>
+        <v>2840.5047</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="19" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="B24" s="19" t="inlineStr">
         <is>
-          <t>Invesco India Liquid Fund - Direct Plan - Growth</t>
+          <t>ICICI Prudential Liquid Fund - Direct Plan - Growth</t>
         </is>
       </c>
       <c r="C24" s="26" t="n">
-        <v>46.6</v>
+        <v>46.5</v>
       </c>
       <c r="D24" s="22" t="n">
-        <v>6.5</v>
+        <v>6.46</v>
       </c>
       <c r="E24" s="22" t="n">
-        <v>6.94</v>
+        <v>6.93</v>
       </c>
       <c r="F24" s="22" t="n">
         <v>6.36</v>
       </c>
       <c r="G24" s="22" t="n">
-        <v>6.09</v>
+        <v>6.11</v>
       </c>
       <c r="H24" s="22" t="n">
-        <v>6.74</v>
+        <v>6.71</v>
       </c>
       <c r="I24" s="22" t="n">
+        <v>6.75</v>
+      </c>
+      <c r="J24" s="22" t="n">
         <v>6.76</v>
       </c>
-      <c r="J24" s="22" t="n">
-        <v>6.74</v>
-      </c>
       <c r="K24" s="22" t="n">
-        <v>6.5</v>
+        <v>6.52</v>
       </c>
       <c r="L24" s="23" t="n">
-        <v>-13.73</v>
+        <v>-13.72</v>
       </c>
       <c r="M24" s="23" t="n"/>
       <c r="N24" s="23" t="n">
         <v>0.13</v>
       </c>
       <c r="O24" s="23" t="n">
-        <v>-0.23</v>
+        <v>-0.16</v>
       </c>
       <c r="P24" s="23" t="n">
-        <v>30.17</v>
+        <v>43.31</v>
       </c>
       <c r="Q24" s="23" t="n">
         <v>0.01</v>
@@ -53018,7 +53020,7 @@
         <v>-6.1</v>
       </c>
       <c r="T24" s="22" t="n">
-        <v>4.82</v>
+        <v>4.83</v>
       </c>
       <c r="U24" s="25" t="n">
         <v>0.001</v>
@@ -53027,66 +53029,66 @@
         <v>0.006</v>
       </c>
       <c r="W24" s="21" t="n">
-        <v>-0.11</v>
+        <v>-0.12</v>
       </c>
       <c r="X24" s="24" t="n">
         <v>100</v>
       </c>
       <c r="Y24" s="24" t="n">
-        <v>13.7</v>
+        <v>13.8</v>
       </c>
       <c r="Z24" s="19" t="n">
-        <v>3911.4333</v>
+        <v>421.8632</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="7" t="n">
-        <v>23</v>
+        <v>18</v>
       </c>
       <c r="B25" s="7" t="inlineStr">
         <is>
-          <t>SBI Liquid Fund - DIRECT PLAN -Growth</t>
+          <t>Invesco India Liquid Fund - Direct Plan - Growth</t>
         </is>
       </c>
       <c r="C25" s="27" t="n">
         <v>46.5</v>
       </c>
       <c r="D25" s="11" t="n">
-        <v>6.47</v>
+        <v>6.5</v>
       </c>
       <c r="E25" s="11" t="n">
-        <v>6.89</v>
+        <v>6.93</v>
       </c>
       <c r="F25" s="11" t="n">
-        <v>6.34</v>
+        <v>6.37</v>
       </c>
       <c r="G25" s="11" t="n">
-        <v>6.07</v>
+        <v>6.08</v>
       </c>
       <c r="H25" s="11" t="n">
-        <v>6.69</v>
+        <v>6.73</v>
       </c>
       <c r="I25" s="11" t="n">
-        <v>6.72</v>
+        <v>6.76</v>
       </c>
       <c r="J25" s="11" t="n">
-        <v>6.71</v>
+        <v>6.74</v>
       </c>
       <c r="K25" s="11" t="n">
-        <v>6.47</v>
+        <v>6.5</v>
       </c>
       <c r="L25" s="9" t="n">
-        <v>-13.91</v>
+        <v>-13.75</v>
       </c>
       <c r="M25" s="9" t="n"/>
       <c r="N25" s="9" t="n">
         <v>0.13</v>
       </c>
       <c r="O25" s="9" t="n">
-        <v>-0.17</v>
+        <v>-0.23</v>
       </c>
       <c r="P25" s="9" t="n">
-        <v>40.53</v>
+        <v>30.13</v>
       </c>
       <c r="Q25" s="9" t="n">
         <v>0.01</v>
@@ -53095,80 +53097,80 @@
         <v>1.4</v>
       </c>
       <c r="S25" s="17" t="n">
-        <v>-6</v>
+        <v>-6.1</v>
       </c>
       <c r="T25" s="11" t="n">
-        <v>4.8</v>
+        <v>4.82</v>
       </c>
       <c r="U25" s="18" t="n">
         <v>0.001</v>
       </c>
       <c r="V25" s="18" t="n">
-        <v>0.008</v>
+        <v>0.007</v>
       </c>
       <c r="W25" s="10" t="n">
-        <v>-0.11</v>
+        <v>-0.13</v>
       </c>
       <c r="X25" s="17" t="n">
         <v>100</v>
       </c>
       <c r="Y25" s="17" t="n">
-        <v>13.7</v>
+        <v>13.8</v>
       </c>
       <c r="Z25" s="7" t="n">
-        <v>4454.3239</v>
+        <v>3913.3296</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="19" t="n">
-        <v>23</v>
+        <v>18</v>
       </c>
       <c r="B26" s="19" t="inlineStr">
         <is>
-          <t>BANDHAN LIQUID Fund -Direct Plan-Growth</t>
+          <t>Mirae Asset Liquid Fund - Direct Plan - Growth</t>
         </is>
       </c>
       <c r="C26" s="26" t="n">
         <v>46.5</v>
       </c>
       <c r="D26" s="22" t="n">
-        <v>6.48</v>
+        <v>6.43</v>
       </c>
       <c r="E26" s="22" t="n">
         <v>6.92</v>
       </c>
       <c r="F26" s="22" t="n">
-        <v>6.37</v>
+        <v>6.38</v>
       </c>
       <c r="G26" s="22" t="n">
-        <v>6.05</v>
+        <v>6.11</v>
       </c>
       <c r="H26" s="22" t="n">
-        <v>6.71</v>
+        <v>6.7</v>
       </c>
       <c r="I26" s="22" t="n">
         <v>6.75</v>
       </c>
       <c r="J26" s="22" t="n">
-        <v>6.7</v>
+        <v>6.66</v>
       </c>
       <c r="K26" s="22" t="n">
-        <v>6.46</v>
+        <v>6.45</v>
       </c>
       <c r="L26" s="23" t="n">
-        <v>-13.82</v>
+        <v>-14.42</v>
       </c>
       <c r="M26" s="23" t="n">
-        <v>-45.79</v>
+        <v>-23.14</v>
       </c>
       <c r="N26" s="23" t="n">
-        <v>0.13</v>
+        <v>0.12</v>
       </c>
       <c r="O26" s="23" t="n">
-        <v>-0.23</v>
+        <v>-0.16</v>
       </c>
       <c r="P26" s="23" t="n">
-        <v>30.09</v>
+        <v>43.25</v>
       </c>
       <c r="Q26" s="23" t="n">
         <v>0.01</v>
@@ -53180,7 +53182,7 @@
         <v>-6</v>
       </c>
       <c r="T26" s="22" t="n">
-        <v>4.81</v>
+        <v>4.8</v>
       </c>
       <c r="U26" s="25" t="n">
         <v>0.001</v>
@@ -53189,7 +53191,7 @@
         <v>0.006</v>
       </c>
       <c r="W26" s="21" t="n">
-        <v>-0.11</v>
+        <v>-0.13</v>
       </c>
       <c r="X26" s="24" t="n">
         <v>100</v>
@@ -53198,57 +53200,59 @@
         <v>13.7</v>
       </c>
       <c r="Z26" s="19" t="n">
-        <v>3440.6675</v>
+        <v>3009.7282</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="7" t="n">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="B27" s="7" t="inlineStr">
         <is>
-          <t>JM Liquid Fund (Direct) - Growth Option</t>
+          <t>CANARA ROBECO LIQUID FUND - DIRECT PLAN - GROWTH OPTION</t>
         </is>
       </c>
       <c r="C27" s="27" t="n">
-        <v>46.5</v>
+        <v>46.4</v>
       </c>
       <c r="D27" s="11" t="n">
-        <v>6.39</v>
+        <v>6.46</v>
       </c>
       <c r="E27" s="11" t="n">
-        <v>6.85</v>
+        <v>6.94</v>
       </c>
       <c r="F27" s="11" t="n">
-        <v>6.32</v>
+        <v>6.38</v>
       </c>
       <c r="G27" s="11" t="n">
-        <v>6.08</v>
+        <v>5.99</v>
       </c>
       <c r="H27" s="11" t="n">
-        <v>6.64</v>
+        <v>6.73</v>
       </c>
       <c r="I27" s="11" t="n">
-        <v>6.69</v>
+        <v>6.77</v>
       </c>
       <c r="J27" s="11" t="n">
-        <v>6.76</v>
+        <v>6.63</v>
       </c>
       <c r="K27" s="11" t="n">
-        <v>6.52</v>
+        <v>6.38</v>
       </c>
       <c r="L27" s="9" t="n">
-        <v>-7.78</v>
-      </c>
-      <c r="M27" s="9" t="n"/>
+        <v>-13.93</v>
+      </c>
+      <c r="M27" s="9" t="n">
+        <v>-28.07</v>
+      </c>
       <c r="N27" s="9" t="n">
-        <v>0.16</v>
+        <v>0.12</v>
       </c>
       <c r="O27" s="9" t="n">
         <v>-0.18</v>
       </c>
       <c r="P27" s="9" t="n">
-        <v>38.06</v>
+        <v>38.56</v>
       </c>
       <c r="Q27" s="9" t="n">
         <v>0.01</v>
@@ -53260,77 +53264,75 @@
         <v>-6</v>
       </c>
       <c r="T27" s="11" t="n">
-        <v>4.78</v>
+        <v>4.81</v>
       </c>
       <c r="U27" s="18" t="n">
         <v>0.001</v>
       </c>
       <c r="V27" s="18" t="n">
-        <v>0.008999999999999999</v>
+        <v>0.008</v>
       </c>
       <c r="W27" s="10" t="n">
-        <v>-0.11</v>
+        <v>-0.13</v>
       </c>
       <c r="X27" s="17" t="n">
         <v>100</v>
       </c>
       <c r="Y27" s="17" t="n">
-        <v>13.7</v>
+        <v>13.8</v>
       </c>
       <c r="Z27" s="7" t="n">
-        <v>77.7269</v>
+        <v>3416.7965</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="19" t="n">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="B28" s="19" t="inlineStr">
         <is>
-          <t>Mirae Asset Liquid Fund - Direct Plan - Growth</t>
+          <t>SBI Liquid Fund - DIRECT PLAN -Growth</t>
         </is>
       </c>
       <c r="C28" s="26" t="n">
-        <v>46.5</v>
+        <v>46.4</v>
       </c>
       <c r="D28" s="22" t="n">
-        <v>6.43</v>
+        <v>6.47</v>
       </c>
       <c r="E28" s="22" t="n">
-        <v>6.93</v>
+        <v>6.89</v>
       </c>
       <c r="F28" s="22" t="n">
-        <v>6.38</v>
+        <v>6.35</v>
       </c>
       <c r="G28" s="22" t="n">
-        <v>6.11</v>
+        <v>6.06</v>
       </c>
       <c r="H28" s="22" t="n">
-        <v>6.7</v>
+        <v>6.69</v>
       </c>
       <c r="I28" s="22" t="n">
-        <v>6.75</v>
+        <v>6.72</v>
       </c>
       <c r="J28" s="22" t="n">
-        <v>6.66</v>
+        <v>6.71</v>
       </c>
       <c r="K28" s="22" t="n">
-        <v>6.45</v>
+        <v>6.47</v>
       </c>
       <c r="L28" s="23" t="n">
-        <v>-14.4</v>
-      </c>
-      <c r="M28" s="23" t="n">
-        <v>-23.1</v>
-      </c>
+        <v>-13.93</v>
+      </c>
+      <c r="M28" s="23" t="n"/>
       <c r="N28" s="23" t="n">
-        <v>0.12</v>
+        <v>0.13</v>
       </c>
       <c r="O28" s="23" t="n">
-        <v>-0.16</v>
+        <v>-0.17</v>
       </c>
       <c r="P28" s="23" t="n">
-        <v>43.31</v>
+        <v>40.53</v>
       </c>
       <c r="Q28" s="23" t="n">
         <v>0.01</v>
@@ -53339,7 +53341,7 @@
         <v>1.4</v>
       </c>
       <c r="S28" s="24" t="n">
-        <v>-6.1</v>
+        <v>-6</v>
       </c>
       <c r="T28" s="22" t="n">
         <v>4.8</v>
@@ -53348,71 +53350,69 @@
         <v>0.001</v>
       </c>
       <c r="V28" s="25" t="n">
-        <v>0.006</v>
+        <v>0.008</v>
       </c>
       <c r="W28" s="21" t="n">
-        <v>-0.11</v>
+        <v>-0.13</v>
       </c>
       <c r="X28" s="24" t="n">
         <v>100</v>
       </c>
       <c r="Y28" s="24" t="n">
-        <v>13.7</v>
+        <v>13.8</v>
       </c>
       <c r="Z28" s="19" t="n">
-        <v>3008.2407</v>
+        <v>4456.4395</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="7" t="n">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="B29" s="7" t="inlineStr">
         <is>
-          <t>CANARA ROBECO LIQUID FUND - DIRECT PLAN - GROWTH OPTION</t>
+          <t>JM Liquid Fund (Direct) - Growth Option</t>
         </is>
       </c>
       <c r="C29" s="27" t="n">
         <v>46.4</v>
       </c>
       <c r="D29" s="11" t="n">
-        <v>6.46</v>
+        <v>6.39</v>
       </c>
       <c r="E29" s="11" t="n">
-        <v>6.94</v>
+        <v>6.85</v>
       </c>
       <c r="F29" s="11" t="n">
-        <v>6.38</v>
+        <v>6.33</v>
       </c>
       <c r="G29" s="11" t="n">
-        <v>5.99</v>
+        <v>6.08</v>
       </c>
       <c r="H29" s="11" t="n">
-        <v>6.73</v>
+        <v>6.64</v>
       </c>
       <c r="I29" s="11" t="n">
-        <v>6.77</v>
+        <v>6.69</v>
       </c>
       <c r="J29" s="11" t="n">
-        <v>6.64</v>
+        <v>6.76</v>
       </c>
       <c r="K29" s="11" t="n">
-        <v>6.38</v>
+        <v>6.52</v>
       </c>
       <c r="L29" s="9" t="n">
-        <v>-13.92</v>
-      </c>
-      <c r="M29" s="9" t="n">
-        <v>-28.04</v>
-      </c>
+        <v>-7.8</v>
+      </c>
+      <c r="M29" s="9" t="n"/>
       <c r="N29" s="9" t="n">
-        <v>0.12</v>
+        <v>0.16</v>
       </c>
       <c r="O29" s="9" t="n">
         <v>-0.18</v>
       </c>
       <c r="P29" s="9" t="n">
-        <v>38.56</v>
+        <v>38.06</v>
       </c>
       <c r="Q29" s="9" t="n">
         <v>0.01</v>
@@ -53424,13 +53424,13 @@
         <v>-6</v>
       </c>
       <c r="T29" s="11" t="n">
-        <v>4.81</v>
+        <v>4.78</v>
       </c>
       <c r="U29" s="18" t="n">
         <v>0.001</v>
       </c>
       <c r="V29" s="18" t="n">
-        <v>0.008</v>
+        <v>0.01</v>
       </c>
       <c r="W29" s="10" t="n">
         <v>-0.13</v>
@@ -53439,10 +53439,10 @@
         <v>100</v>
       </c>
       <c r="Y29" s="17" t="n">
-        <v>13.7</v>
+        <v>13.8</v>
       </c>
       <c r="Z29" s="7" t="n">
-        <v>3415.6728</v>
+        <v>77.7645</v>
       </c>
     </row>
     <row r="30">
@@ -53458,13 +53458,13 @@
         <v>46.3</v>
       </c>
       <c r="D30" s="22" t="n">
-        <v>6.5</v>
+        <v>6.49</v>
       </c>
       <c r="E30" s="22" t="n">
         <v>6.95</v>
       </c>
       <c r="F30" s="22" t="n">
-        <v>6.4</v>
+        <v>6.41</v>
       </c>
       <c r="G30" s="22" t="n">
         <v>5.73</v>
@@ -53482,7 +53482,7 @@
         <v>6.14</v>
       </c>
       <c r="L30" s="23" t="n">
-        <v>-14.68</v>
+        <v>-14.7</v>
       </c>
       <c r="M30" s="23" t="n"/>
       <c r="N30" s="23" t="n">
@@ -53504,7 +53504,7 @@
         <v>-6.1</v>
       </c>
       <c r="T30" s="22" t="n">
-        <v>4.83</v>
+        <v>4.82</v>
       </c>
       <c r="U30" s="25" t="n">
         <v>0.001</v>
@@ -53513,16 +53513,16 @@
         <v>0.006</v>
       </c>
       <c r="W30" s="21" t="n">
-        <v>-0.11</v>
+        <v>-0.13</v>
       </c>
       <c r="X30" s="24" t="n">
         <v>100</v>
       </c>
       <c r="Y30" s="24" t="n">
-        <v>13.7</v>
+        <v>13.8</v>
       </c>
       <c r="Z30" s="19" t="n">
-        <v>2748.6839</v>
+        <v>2750.0301</v>
       </c>
     </row>
     <row r="31">
@@ -53541,10 +53541,10 @@
         <v>6.52</v>
       </c>
       <c r="E31" s="11" t="n">
-        <v>6.97</v>
+        <v>6.96</v>
       </c>
       <c r="F31" s="11" t="n">
-        <v>6.42</v>
+        <v>6.43</v>
       </c>
       <c r="G31" s="11" t="n">
         <v>6.19</v>
@@ -53559,10 +53559,10 @@
         <v>6.15</v>
       </c>
       <c r="K31" s="11" t="n">
-        <v>5.92</v>
+        <v>5.93</v>
       </c>
       <c r="L31" s="9" t="n">
-        <v>-14.93</v>
+        <v>-14.94</v>
       </c>
       <c r="M31" s="9" t="n"/>
       <c r="N31" s="9" t="n">
@@ -53572,7 +53572,7 @@
         <v>-0.22</v>
       </c>
       <c r="P31" s="9" t="n">
-        <v>31.68</v>
+        <v>31.64</v>
       </c>
       <c r="Q31" s="9" t="n">
         <v>0.01</v>
@@ -53593,16 +53593,16 @@
         <v>0.008</v>
       </c>
       <c r="W31" s="10" t="n">
-        <v>-0.11</v>
+        <v>-0.13</v>
       </c>
       <c r="X31" s="17" t="n">
         <v>100</v>
       </c>
       <c r="Y31" s="17" t="n">
-        <v>10.2</v>
+        <v>10.3</v>
       </c>
       <c r="Z31" s="7" t="n">
-        <v>1856.502</v>
+        <v>1857.3939</v>
       </c>
     </row>
     <row r="32">
@@ -53621,7 +53621,7 @@
         <v>6.51</v>
       </c>
       <c r="E32" s="22" t="n">
-        <v>6.97</v>
+        <v>6.96</v>
       </c>
       <c r="F32" s="22" t="n">
         <v>6.41</v>
@@ -53630,10 +53630,10 @@
         <v>6.16</v>
       </c>
       <c r="H32" s="22" t="n">
-        <v>6.77</v>
+        <v>6.76</v>
       </c>
       <c r="I32" s="22" t="n">
-        <v>6.8</v>
+        <v>6.79</v>
       </c>
       <c r="J32" s="22" t="n">
         <v>6.16</v>
@@ -53642,7 +53642,7 @@
         <v>5.95</v>
       </c>
       <c r="L32" s="23" t="n">
-        <v>-13.05</v>
+        <v>-13.07</v>
       </c>
       <c r="M32" s="23" t="n"/>
       <c r="N32" s="23" t="n">
@@ -53652,7 +53652,7 @@
         <v>-0.15</v>
       </c>
       <c r="P32" s="23" t="n">
-        <v>46.47</v>
+        <v>46.4</v>
       </c>
       <c r="Q32" s="23" t="n">
         <v>0.01</v>
@@ -53673,7 +53673,7 @@
         <v>0.006</v>
       </c>
       <c r="W32" s="21" t="n">
-        <v>-0.11</v>
+        <v>-0.12</v>
       </c>
       <c r="X32" s="24" t="n">
         <v>100</v>
@@ -53682,7 +53682,7 @@
         <v>10.6</v>
       </c>
       <c r="Z32" s="19" t="n">
-        <v>371.866</v>
+        <v>372.0402</v>
       </c>
     </row>
     <row r="33">
@@ -53691,48 +53691,48 @@
       </c>
       <c r="B33" s="7" t="inlineStr">
         <is>
-          <t>360 ONE LIQUID FUND DIRECT PLAN  GROWTH</t>
+          <t>Sundaram Liquid Fund (Formerly Known as Principal Cash Management Fund) - Direct Plan - Growth Option</t>
         </is>
       </c>
       <c r="C33" s="27" t="n">
         <v>45.9</v>
       </c>
       <c r="D33" s="11" t="n">
-        <v>6.28</v>
+        <v>6.56</v>
       </c>
       <c r="E33" s="11" t="n">
-        <v>6.74</v>
+        <v>6.98</v>
       </c>
       <c r="F33" s="11" t="n">
-        <v>6.2</v>
+        <v>6.24</v>
       </c>
       <c r="G33" s="11" t="n">
-        <v>5.73</v>
+        <v>3.07</v>
       </c>
       <c r="H33" s="11" t="n">
-        <v>6.53</v>
+        <v>6.79</v>
       </c>
       <c r="I33" s="11" t="n">
-        <v>6.58</v>
+        <v>6.85</v>
       </c>
       <c r="J33" s="11" t="n">
-        <v>6.14</v>
+        <v>6.87</v>
       </c>
       <c r="K33" s="11" t="n">
-        <v>5.89</v>
+        <v>6.99</v>
       </c>
       <c r="L33" s="9" t="n">
-        <v>-5.1</v>
+        <v>-12.76</v>
       </c>
       <c r="M33" s="9" t="n"/>
       <c r="N33" s="9" t="n">
-        <v>0.18</v>
+        <v>0.13</v>
       </c>
       <c r="O33" s="9" t="n">
-        <v>-0.04</v>
+        <v>-0.02</v>
       </c>
       <c r="P33" s="9" t="n">
-        <v>168.5</v>
+        <v>349</v>
       </c>
       <c r="Q33" s="9" t="n">
         <v>0.01</v>
@@ -53741,16 +53741,16 @@
         <v>1.4</v>
       </c>
       <c r="S33" s="17" t="n">
-        <v>-6</v>
+        <v>-6.1</v>
       </c>
       <c r="T33" s="11" t="n">
-        <v>4.73</v>
+        <v>4.86</v>
       </c>
       <c r="U33" s="18" t="n">
         <v>0.001</v>
       </c>
       <c r="V33" s="18" t="n">
-        <v>0.01</v>
+        <v>0.008</v>
       </c>
       <c r="W33" s="10" t="n">
         <v>-0.12</v>
@@ -53759,170 +53759,170 @@
         <v>100</v>
       </c>
       <c r="Y33" s="17" t="n">
-        <v>12.9</v>
+        <v>4.8</v>
       </c>
       <c r="Z33" s="7" t="n">
-        <v>2180.7113</v>
+        <v>2520.969</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="19" t="n">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B34" s="19" t="inlineStr">
         <is>
-          <t>Sundaram Liquid Fund (Formerly Known as Principal Cash Management Fund) - Direct Plan - Growth Option</t>
+          <t>Quantum Liquid Fund - Direct Plan Growth Option</t>
         </is>
       </c>
       <c r="C34" s="26" t="n">
-        <v>45.9</v>
+        <v>45.8</v>
       </c>
       <c r="D34" s="22" t="n">
-        <v>6.57</v>
+        <v>5.93</v>
       </c>
       <c r="E34" s="22" t="n">
-        <v>6.99</v>
+        <v>6.51</v>
       </c>
       <c r="F34" s="22" t="n">
-        <v>6.23</v>
+        <v>6.04</v>
       </c>
       <c r="G34" s="22" t="n">
-        <v>3.07</v>
+        <v>5.64</v>
       </c>
       <c r="H34" s="22" t="n">
-        <v>6.8</v>
+        <v>6.24</v>
       </c>
       <c r="I34" s="22" t="n">
-        <v>6.85</v>
+        <v>6.35</v>
       </c>
       <c r="J34" s="22" t="n">
-        <v>6.87</v>
+        <v>6.73</v>
       </c>
       <c r="K34" s="22" t="n">
-        <v>6.99</v>
+        <v>6.68</v>
       </c>
       <c r="L34" s="23" t="n">
-        <v>-12.74</v>
+        <v>-22.76</v>
       </c>
       <c r="M34" s="23" t="n"/>
       <c r="N34" s="23" t="n">
-        <v>0.13</v>
+        <v>0.09</v>
       </c>
       <c r="O34" s="23" t="n">
-        <v>-0.02</v>
+        <v>-0.55</v>
       </c>
       <c r="P34" s="23" t="n">
-        <v>349.5</v>
+        <v>11.84</v>
       </c>
       <c r="Q34" s="23" t="n">
         <v>0.01</v>
       </c>
       <c r="R34" s="24" t="n">
-        <v>1.4</v>
+        <v>1.3</v>
       </c>
       <c r="S34" s="24" t="n">
-        <v>-6.1</v>
+        <v>-5.7</v>
       </c>
       <c r="T34" s="22" t="n">
-        <v>4.87</v>
+        <v>4.48</v>
       </c>
       <c r="U34" s="25" t="n">
         <v>0.001</v>
       </c>
       <c r="V34" s="25" t="n">
-        <v>0.008</v>
+        <v>0.007</v>
       </c>
       <c r="W34" s="21" t="n">
-        <v>-0.11</v>
+        <v>-0.15</v>
       </c>
       <c r="X34" s="24" t="n">
         <v>100</v>
       </c>
       <c r="Y34" s="24" t="n">
-        <v>4.7</v>
+        <v>20.5</v>
       </c>
       <c r="Z34" s="19" t="n">
-        <v>2519.7578</v>
+        <v>37.8612</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="7" t="n">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="B35" s="7" t="inlineStr">
         <is>
-          <t>Quantum Liquid Fund - Direct Plan Growth Option</t>
+          <t>360 ONE LIQUID FUND DIRECT PLAN  GROWTH</t>
         </is>
       </c>
       <c r="C35" s="27" t="n">
         <v>45.8</v>
       </c>
       <c r="D35" s="11" t="n">
-        <v>5.93</v>
+        <v>6.27</v>
       </c>
       <c r="E35" s="11" t="n">
-        <v>6.51</v>
+        <v>6.74</v>
       </c>
       <c r="F35" s="11" t="n">
-        <v>6.04</v>
+        <v>6.2</v>
       </c>
       <c r="G35" s="11" t="n">
-        <v>5.64</v>
+        <v>5.73</v>
       </c>
       <c r="H35" s="11" t="n">
-        <v>6.24</v>
+        <v>6.53</v>
       </c>
       <c r="I35" s="11" t="n">
-        <v>6.35</v>
+        <v>6.58</v>
       </c>
       <c r="J35" s="11" t="n">
-        <v>6.74</v>
+        <v>6.14</v>
       </c>
       <c r="K35" s="11" t="n">
-        <v>6.68</v>
+        <v>5.89</v>
       </c>
       <c r="L35" s="9" t="n">
-        <v>-22.75</v>
+        <v>-5.01</v>
       </c>
       <c r="M35" s="9" t="n"/>
       <c r="N35" s="9" t="n">
-        <v>0.09</v>
+        <v>0.18</v>
       </c>
       <c r="O35" s="9" t="n">
-        <v>-0.55</v>
+        <v>-0.04</v>
       </c>
       <c r="P35" s="9" t="n">
-        <v>11.84</v>
+        <v>168.5</v>
       </c>
       <c r="Q35" s="9" t="n">
         <v>0.01</v>
       </c>
       <c r="R35" s="17" t="n">
-        <v>1.3</v>
+        <v>1.4</v>
       </c>
       <c r="S35" s="17" t="n">
-        <v>-5.7</v>
+        <v>-6</v>
       </c>
       <c r="T35" s="11" t="n">
-        <v>4.48</v>
+        <v>4.73</v>
       </c>
       <c r="U35" s="18" t="n">
         <v>0.001</v>
       </c>
       <c r="V35" s="18" t="n">
-        <v>0.007</v>
+        <v>0.01</v>
       </c>
       <c r="W35" s="10" t="n">
-        <v>-0.15</v>
+        <v>-0.13</v>
       </c>
       <c r="X35" s="17" t="n">
         <v>100</v>
       </c>
       <c r="Y35" s="17" t="n">
-        <v>20.5</v>
+        <v>12.9</v>
       </c>
       <c r="Z35" s="7" t="n">
-        <v>37.8494</v>
+        <v>2181.8699</v>
       </c>
     </row>
     <row r="36">
@@ -53941,13 +53941,13 @@
         <v>6.43</v>
       </c>
       <c r="E36" s="22" t="n">
-        <v>6.88</v>
+        <v>6.87</v>
       </c>
       <c r="F36" s="22" t="n">
-        <v>6.33</v>
+        <v>6.34</v>
       </c>
       <c r="G36" s="22" t="n">
-        <v>3.26</v>
+        <v>3.27</v>
       </c>
       <c r="H36" s="22" t="n">
         <v>6.67</v>
@@ -53962,7 +53962,7 @@
         <v>6.66</v>
       </c>
       <c r="L36" s="23" t="n">
-        <v>-11.66</v>
+        <v>-11.68</v>
       </c>
       <c r="M36" s="23" t="n"/>
       <c r="N36" s="23" t="n">
@@ -53972,7 +53972,7 @@
         <v>-0.01</v>
       </c>
       <c r="P36" s="23" t="n">
-        <v>688</v>
+        <v>687</v>
       </c>
       <c r="Q36" s="23" t="n">
         <v>0.01</v>
@@ -53993,7 +53993,7 @@
         <v>0.008999999999999999</v>
       </c>
       <c r="W36" s="21" t="n">
-        <v>-0.11</v>
+        <v>-0.13</v>
       </c>
       <c r="X36" s="24" t="n">
         <v>100</v>
@@ -54002,7 +54002,7 @@
         <v>5.4</v>
       </c>
       <c r="Z36" s="19" t="n">
-        <v>1379.1587</v>
+        <v>1379.8256</v>
       </c>
     </row>
     <row r="37">
@@ -54097,22 +54097,22 @@
         </is>
       </c>
       <c r="C38" s="26" t="n">
-        <v>45.3</v>
+        <v>45.2</v>
       </c>
       <c r="D38" s="22" t="n">
-        <v>6.41</v>
+        <v>6.39</v>
       </c>
       <c r="E38" s="22" t="n">
-        <v>6.85</v>
+        <v>6.84</v>
       </c>
       <c r="F38" s="22" t="n">
-        <v>6.21</v>
+        <v>6.22</v>
       </c>
       <c r="G38" s="22" t="n">
         <v>4.31</v>
       </c>
       <c r="H38" s="22" t="n">
-        <v>6.65</v>
+        <v>6.64</v>
       </c>
       <c r="I38" s="22" t="n">
         <v>6.65</v>
@@ -54121,20 +54121,20 @@
         <v>5.46</v>
       </c>
       <c r="K38" s="22" t="n">
-        <v>5.4</v>
+        <v>5.41</v>
       </c>
       <c r="L38" s="23" t="n">
-        <v>-4.49</v>
+        <v>-4.42</v>
       </c>
       <c r="M38" s="23" t="n"/>
       <c r="N38" s="23" t="n">
-        <v>0.18</v>
+        <v>0.19</v>
       </c>
       <c r="O38" s="23" t="n">
         <v>-0.05</v>
       </c>
       <c r="P38" s="23" t="n">
-        <v>137</v>
+        <v>136.8</v>
       </c>
       <c r="Q38" s="23" t="n">
         <v>0.01</v>
@@ -54155,7 +54155,7 @@
         <v>0.008</v>
       </c>
       <c r="W38" s="21" t="n">
-        <v>-0.11</v>
+        <v>-0.13</v>
       </c>
       <c r="X38" s="24" t="n">
         <v>100</v>
@@ -54164,7 +54164,7 @@
         <v>7.7</v>
       </c>
       <c r="Z38" s="19" t="n">
-        <v>1525.2315</v>
+        <v>1525.9649</v>
       </c>
     </row>
     <row r="39">
@@ -54186,10 +54186,10 @@
         <v>6.69</v>
       </c>
       <c r="F39" s="11" t="n">
-        <v>6.1</v>
+        <v>6.11</v>
       </c>
       <c r="G39" s="11" t="n">
-        <v>4.64</v>
+        <v>4.65</v>
       </c>
       <c r="H39" s="11" t="n">
         <v>6.56</v>
@@ -54201,13 +54201,13 @@
         <v>5.44</v>
       </c>
       <c r="K39" s="11" t="n">
-        <v>5.23</v>
+        <v>5.24</v>
       </c>
       <c r="L39" s="9" t="n">
-        <v>-15.09</v>
+        <v>-15.1</v>
       </c>
       <c r="M39" s="9" t="n">
-        <v>-20.26</v>
+        <v>-20.27</v>
       </c>
       <c r="N39" s="9" t="n">
         <v>0.12</v>
@@ -54246,7 +54246,7 @@
         <v>8.4</v>
       </c>
       <c r="Z39" s="7" t="n">
-        <v>1575.7675</v>
+        <v>1576.2833</v>
       </c>
     </row>
     <row r="40">
@@ -54268,25 +54268,25 @@
         <v>6.68</v>
       </c>
       <c r="F40" s="22" t="n">
-        <v>6.14</v>
+        <v>6.15</v>
       </c>
       <c r="G40" s="22" t="n">
-        <v>3.98</v>
+        <v>3.99</v>
       </c>
       <c r="H40" s="22" t="n">
-        <v>6.48</v>
+        <v>6.47</v>
       </c>
       <c r="I40" s="22" t="n">
         <v>6.51</v>
       </c>
       <c r="J40" s="22" t="n">
-        <v>5.32</v>
+        <v>5.33</v>
       </c>
       <c r="K40" s="22" t="n">
         <v>5.43</v>
       </c>
       <c r="L40" s="23" t="n">
-        <v>-16.58</v>
+        <v>-16.6</v>
       </c>
       <c r="M40" s="23" t="n"/>
       <c r="N40" s="23" t="n">
@@ -54317,7 +54317,7 @@
         <v>0.003</v>
       </c>
       <c r="W40" s="21" t="n">
-        <v>-0.12</v>
+        <v>-0.14</v>
       </c>
       <c r="X40" s="24" t="n">
         <v>100</v>
@@ -54326,7 +54326,7 @@
         <v>7.4</v>
       </c>
       <c r="Z40" s="19" t="n">
-        <v>1477.9439</v>
+        <v>1478.636</v>
       </c>
     </row>
     <row r="41">
@@ -54339,10 +54339,10 @@
         </is>
       </c>
       <c r="C41" s="27" t="n">
-        <v>44.7</v>
+        <v>44.6</v>
       </c>
       <c r="D41" s="11" t="n">
-        <v>6.11</v>
+        <v>6.09</v>
       </c>
       <c r="E41" s="11" t="n">
         <v>6.55</v>
@@ -54351,7 +54351,7 @@
         <v>6</v>
       </c>
       <c r="G41" s="11" t="n">
-        <v>4.13</v>
+        <v>4.14</v>
       </c>
       <c r="H41" s="11" t="n">
         <v>6.33</v>
@@ -54366,7 +54366,7 @@
         <v>5.22</v>
       </c>
       <c r="L41" s="9" t="n">
-        <v>-6.56</v>
+        <v>-6.47</v>
       </c>
       <c r="M41" s="9" t="n"/>
       <c r="N41" s="9" t="n">
@@ -54397,7 +54397,7 @@
         <v>0.012</v>
       </c>
       <c r="W41" s="10" t="n">
-        <v>-0.13</v>
+        <v>-0.14</v>
       </c>
       <c r="X41" s="17" t="n">
         <v>100</v>
@@ -54406,7 +54406,7 @@
         <v>7.8</v>
       </c>
       <c r="Z41" s="7" t="n">
-        <v>14.9959</v>
+        <v>15.0027</v>
       </c>
     </row>
     <row r="42">
@@ -54422,22 +54422,22 @@
         <v>43.3</v>
       </c>
       <c r="D42" s="22" t="n">
-        <v>6.08</v>
+        <v>6.07</v>
       </c>
       <c r="E42" s="22" t="n">
-        <v>6.75</v>
+        <v>6.74</v>
       </c>
       <c r="F42" s="22" t="n">
-        <v>6.3</v>
+        <v>6.31</v>
       </c>
       <c r="G42" s="22" t="n">
-        <v>6.34</v>
+        <v>6.33</v>
       </c>
       <c r="H42" s="22" t="n">
         <v>6.48</v>
       </c>
       <c r="I42" s="22" t="n">
-        <v>6.58</v>
+        <v>6.57</v>
       </c>
       <c r="J42" s="22" t="n">
         <v>7.03</v>
@@ -54446,7 +54446,7 @@
         <v>6.84</v>
       </c>
       <c r="L42" s="23" t="n">
-        <v>-5.56</v>
+        <v>-5.5</v>
       </c>
       <c r="M42" s="23" t="n"/>
       <c r="N42" s="23" t="n">
@@ -54474,10 +54474,10 @@
         <v>0.001</v>
       </c>
       <c r="V42" s="25" t="n">
-        <v>0.007</v>
+        <v>0.008</v>
       </c>
       <c r="W42" s="21" t="n">
-        <v>-0.12</v>
+        <v>-0.13</v>
       </c>
       <c r="X42" s="24" t="n">
         <v>99.7</v>
@@ -54486,7 +54486,7 @@
         <v>13.7</v>
       </c>
       <c r="Z42" s="19" t="n">
-        <v>45.618</v>
+        <v>45.6381</v>
       </c>
     </row>
     <row r="43">
@@ -54830,29 +54830,29 @@
         <v>41.1</v>
       </c>
       <c r="D47" s="11" t="n">
-        <v>6.57</v>
+        <v>6.56</v>
       </c>
       <c r="E47" s="11" t="n">
-        <v>2.6</v>
+        <v>2.62</v>
       </c>
       <c r="F47" s="11" t="n">
-        <v>1.55</v>
+        <v>1.56</v>
       </c>
       <c r="G47" s="11" t="n">
-        <v>0.77</v>
+        <v>0.78</v>
       </c>
       <c r="H47" s="11" t="n">
-        <v>6.64</v>
+        <v>6.63</v>
       </c>
       <c r="I47" s="11" t="n">
-        <v>6.64</v>
+        <v>6.63</v>
       </c>
       <c r="J47" s="11" t="n">
         <v>6.52</v>
       </c>
       <c r="K47" s="10" t="n"/>
       <c r="L47" s="9" t="n">
-        <v>-12.65</v>
+        <v>-12.7</v>
       </c>
       <c r="M47" s="9" t="n"/>
       <c r="N47" s="9" t="n">
@@ -54862,7 +54862,7 @@
         <v>-0.01</v>
       </c>
       <c r="P47" s="9" t="n">
-        <v>260</v>
+        <v>262</v>
       </c>
       <c r="Q47" s="9" t="n">
         <v>0.01</v>
@@ -54892,7 +54892,7 @@
         <v>1.2</v>
       </c>
       <c r="Z47" s="7" t="n">
-        <v>1080.9481</v>
+        <v>1081.4719</v>
       </c>
     </row>
     <row r="48">
@@ -54905,19 +54905,19 @@
         </is>
       </c>
       <c r="C48" s="26" t="n">
-        <v>40.8</v>
+        <v>40.9</v>
       </c>
       <c r="D48" s="22" t="n">
-        <v>6.32</v>
+        <v>6.33</v>
       </c>
       <c r="E48" s="22" t="n">
-        <v>3.93</v>
+        <v>3.95</v>
       </c>
       <c r="F48" s="22" t="n">
-        <v>2.34</v>
+        <v>2.35</v>
       </c>
       <c r="G48" s="22" t="n">
-        <v>1.16</v>
+        <v>1.17</v>
       </c>
       <c r="H48" s="22" t="n">
         <v>6.33</v>
@@ -54930,10 +54930,10 @@
       </c>
       <c r="K48" s="21" t="n"/>
       <c r="L48" s="23" t="n">
-        <v>-15.33</v>
+        <v>-15.37</v>
       </c>
       <c r="M48" s="23" t="n">
-        <v>-33.25</v>
+        <v>-33.27</v>
       </c>
       <c r="N48" s="23" t="n">
         <v>0.14</v>
@@ -54942,7 +54942,7 @@
         <v>-0.01</v>
       </c>
       <c r="P48" s="23" t="n">
-        <v>393</v>
+        <v>395</v>
       </c>
       <c r="Q48" s="23" t="n">
         <v>0.01</v>
@@ -54972,7 +54972,7 @@
         <v>1.9</v>
       </c>
       <c r="Z48" s="19" t="n">
-        <v>1124.908</v>
+        <v>1125.4576</v>
       </c>
     </row>
     <row r="49">
@@ -55217,7 +55217,7 @@
         </is>
       </c>
       <c r="C52" s="26" t="n">
-        <v>35.9</v>
+        <v>35.8</v>
       </c>
       <c r="D52" s="22" t="n">
         <v>5.76</v>
@@ -55235,16 +55235,16 @@
         <v>6.12</v>
       </c>
       <c r="I52" s="21" t="n">
-        <v>-5.53</v>
+        <v>-5.49</v>
       </c>
       <c r="J52" s="22" t="n">
-        <v>843.11</v>
+        <v>841.85</v>
       </c>
       <c r="K52" s="22" t="n">
-        <v>46.85</v>
+        <v>46.78</v>
       </c>
       <c r="L52" s="23" t="n">
-        <v>-10.99</v>
+        <v>-11</v>
       </c>
       <c r="M52" s="23" t="n"/>
       <c r="N52" s="23" t="n">
@@ -55275,16 +55275,16 @@
         <v>0.015</v>
       </c>
       <c r="W52" s="21" t="n">
-        <v>-0.14</v>
+        <v>-0.15</v>
       </c>
       <c r="X52" s="24" t="n">
         <v>92.2</v>
       </c>
       <c r="Y52" s="24" t="n">
-        <v>13.7</v>
+        <v>13.8</v>
       </c>
       <c r="Z52" s="19" t="n">
-        <v>30.7157</v>
+        <v>30.7299</v>
       </c>
     </row>
     <row r="53">
@@ -55536,29 +55536,29 @@
         <v>34.1</v>
       </c>
       <c r="D56" s="22" t="n">
-        <v>5.84</v>
+        <v>5.83</v>
       </c>
       <c r="E56" s="22" t="n">
-        <v>2.51</v>
+        <v>2.53</v>
       </c>
       <c r="F56" s="22" t="n">
-        <v>1.5</v>
+        <v>1.51</v>
       </c>
       <c r="G56" s="22" t="n">
         <v>0.75</v>
       </c>
       <c r="H56" s="22" t="n">
-        <v>5.79</v>
+        <v>5.78</v>
       </c>
       <c r="I56" s="22" t="n">
-        <v>5.79</v>
+        <v>5.78</v>
       </c>
       <c r="J56" s="22" t="n">
-        <v>5.98</v>
+        <v>5.97</v>
       </c>
       <c r="K56" s="21" t="n"/>
       <c r="L56" s="23" t="n">
-        <v>-16.17</v>
+        <v>-16.24</v>
       </c>
       <c r="M56" s="23" t="n"/>
       <c r="N56" s="23" t="n">
@@ -55596,7 +55596,7 @@
         <v>1.3</v>
       </c>
       <c r="Z56" s="19" t="n">
-        <v>1078.1236</v>
+        <v>1078.5881</v>
       </c>
     </row>
     <row r="57">
@@ -55612,37 +55612,37 @@
         <v>33.9</v>
       </c>
       <c r="D57" s="11" t="n">
-        <v>6.3</v>
+        <v>6.35</v>
       </c>
       <c r="E57" s="11" t="n">
-        <v>2.06</v>
+        <v>2.07</v>
       </c>
       <c r="F57" s="11" t="n">
-        <v>1.23</v>
+        <v>1.24</v>
       </c>
       <c r="G57" s="11" t="n">
-        <v>0.61</v>
+        <v>0.62</v>
       </c>
       <c r="H57" s="11" t="n">
-        <v>6.67</v>
+        <v>6.66</v>
       </c>
       <c r="I57" s="11" t="n">
-        <v>6.67</v>
+        <v>6.66</v>
       </c>
       <c r="J57" s="10" t="n"/>
       <c r="K57" s="10" t="n"/>
       <c r="L57" s="9" t="n">
-        <v>-12.87</v>
+        <v>-12.95</v>
       </c>
       <c r="M57" s="9" t="n"/>
       <c r="N57" s="9" t="n">
-        <v>0.16</v>
+        <v>0.15</v>
       </c>
       <c r="O57" s="9" t="n">
         <v>-0.01</v>
       </c>
       <c r="P57" s="9" t="n">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="Q57" s="9" t="n">
         <v>0.01</v>
@@ -55670,7 +55670,7 @@
         <v>1</v>
       </c>
       <c r="Z57" s="7" t="n">
-        <v>1064.1335</v>
+        <v>1064.6437</v>
       </c>
     </row>
     <row r="58">
@@ -55686,23 +55686,23 @@
         <v>32</v>
       </c>
       <c r="D58" s="22" t="n">
-        <v>5.44</v>
+        <v>5.5</v>
       </c>
       <c r="E58" s="22" t="n">
-        <v>1.78</v>
+        <v>1.8</v>
       </c>
       <c r="F58" s="22" t="n">
-        <v>1.07</v>
+        <v>1.08</v>
       </c>
       <c r="G58" s="22" t="n">
-        <v>0.53</v>
+        <v>0.54</v>
       </c>
       <c r="H58" s="21" t="n"/>
       <c r="I58" s="21" t="n"/>
       <c r="J58" s="21" t="n"/>
       <c r="K58" s="21" t="n"/>
       <c r="L58" s="23" t="n">
-        <v>-13.46</v>
+        <v>-13.55</v>
       </c>
       <c r="M58" s="23" t="n"/>
       <c r="N58" s="23" t="n">
@@ -55712,7 +55712,7 @@
         <v>-0.01</v>
       </c>
       <c r="P58" s="23" t="n">
-        <v>178</v>
+        <v>180</v>
       </c>
       <c r="Q58" s="23" t="n">
         <v>0.01</v>
@@ -55740,7 +55740,7 @@
         <v>0.8</v>
       </c>
       <c r="Z58" s="19" t="n">
-        <v>1056.5021</v>
+        <v>1057.0172</v>
       </c>
     </row>
     <row r="59">
@@ -55756,23 +55756,23 @@
         <v>31.6</v>
       </c>
       <c r="D59" s="11" t="n">
-        <v>4.72</v>
+        <v>4.77</v>
       </c>
       <c r="E59" s="11" t="n">
-        <v>1.55</v>
+        <v>1.56</v>
       </c>
       <c r="F59" s="11" t="n">
-        <v>0.93</v>
+        <v>0.9399999999999999</v>
       </c>
       <c r="G59" s="11" t="n">
-        <v>0.46</v>
+        <v>0.47</v>
       </c>
       <c r="H59" s="10" t="n"/>
       <c r="I59" s="10" t="n"/>
       <c r="J59" s="10" t="n"/>
       <c r="K59" s="10" t="n"/>
       <c r="L59" s="9" t="n">
-        <v>-25.25</v>
+        <v>-25.39</v>
       </c>
       <c r="M59" s="9" t="n"/>
       <c r="N59" s="9" t="n">
@@ -55782,7 +55782,7 @@
         <v>-0.01</v>
       </c>
       <c r="P59" s="9" t="n">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="Q59" s="9" t="n">
         <v>0.01</v>
@@ -55810,7 +55810,7 @@
         <v>0.8</v>
       </c>
       <c r="Z59" s="7" t="n">
-        <v>104.7932</v>
+        <v>104.8417</v>
       </c>
     </row>
     <row r="60">
@@ -55891,7 +55891,7 @@
         </is>
       </c>
       <c r="C61" s="27" t="n">
-        <v>19.4</v>
+        <v>19.3</v>
       </c>
       <c r="D61" s="10" t="n">
         <v>0</v>
@@ -55943,7 +55943,7 @@
       </c>
       <c r="V61" s="18" t="n"/>
       <c r="W61" s="10" t="n">
-        <v>-0.47</v>
+        <v>-0.48</v>
       </c>
       <c r="X61" s="17" t="n">
         <v>0</v>
@@ -55965,7 +55965,7 @@
         </is>
       </c>
       <c r="C62" s="26" t="n">
-        <v>19.4</v>
+        <v>19.3</v>
       </c>
       <c r="D62" s="21" t="n">
         <v>0</v>
@@ -56017,7 +56017,7 @@
       </c>
       <c r="V62" s="25" t="n"/>
       <c r="W62" s="21" t="n">
-        <v>-0.47</v>
+        <v>-0.48</v>
       </c>
       <c r="X62" s="24" t="n">
         <v>0</v>
@@ -56443,7 +56443,7 @@
         <v>-13.7</v>
       </c>
       <c r="T3" s="11" t="n">
-        <v>8427847910015416</v>
+        <v>8427847910015000</v>
       </c>
       <c r="U3" s="18" t="n">
         <v>11.604</v>

</xml_diff>

<commit_message>
🏆 Expert Rankings Updated — 21 Oct 2026 20:45 IST
</commit_message>
<xml_diff>
--- a/output/MF_Expert_Rankings.xlsx
+++ b/output/MF_Expert_Rankings.xlsx
@@ -617,7 +617,7 @@
     <row r="1" ht="50" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>🏆  MF EXPERT RANKINGS  |  Generated: 20 Oct 2026 20:44</t>
+          <t>🏆  MF EXPERT RANKINGS  |  Generated: 21 Oct 2026 20:45</t>
         </is>
       </c>
     </row>
@@ -639,10 +639,10 @@
         </is>
       </c>
       <c r="C4" s="3" t="n">
-        <v>65.90000000000001</v>
+        <v>65.59999999999999</v>
       </c>
       <c r="D4" s="5" t="n">
-        <v>13.09</v>
+        <v>13.03</v>
       </c>
       <c r="E4" s="5" t="n">
         <v>12.01</v>
@@ -654,7 +654,7 @@
         <v>-35.74</v>
       </c>
       <c r="H4" s="7" t="n">
-        <v>9.41</v>
+        <v>9.31</v>
       </c>
     </row>
     <row r="5">
@@ -1170,7 +1170,7 @@
         <v>6.89</v>
       </c>
       <c r="E28" s="10" t="n">
-        <v>6.37</v>
+        <v>6.38</v>
       </c>
       <c r="F28" s="10" t="n">
         <v>-13.05</v>
@@ -1188,26 +1188,26 @@
       </c>
       <c r="B29" s="4" t="inlineStr">
         <is>
-          <t>Kotak Liquid Fund - Direct Plan - Growth</t>
+          <t>LIC MF Liquid Fund-Direct Plan-Growth</t>
         </is>
       </c>
       <c r="C29" s="12" t="n">
         <v>50.1</v>
       </c>
       <c r="D29" s="5" t="n">
-        <v>6.91</v>
+        <v>6.9</v>
       </c>
       <c r="E29" s="5" t="n">
-        <v>6.39</v>
+        <v>6.38</v>
       </c>
       <c r="F29" s="5" t="n">
-        <v>-9.48</v>
+        <v>-13.68</v>
       </c>
       <c r="G29" s="5" t="n">
-        <v>-0.26</v>
+        <v>-0.16</v>
       </c>
       <c r="H29" s="7" t="n">
-        <v>4.83</v>
+        <v>4.79</v>
       </c>
     </row>
     <row r="31">
@@ -1242,7 +1242,7 @@
         <v>-0.42</v>
       </c>
       <c r="H32" s="7" t="n">
-        <v>8427847910015000</v>
+        <v>8427847910015416</v>
       </c>
     </row>
     <row r="33">
@@ -2161,26 +2161,26 @@
       </c>
       <c r="B76" s="4" t="inlineStr">
         <is>
-          <t>Invesco India - Invesco Global Equity Income Fund of Fund - Direct Plan - Growth</t>
+          <t>DSP Global Innovation Overseas Equity Omni FoF - Direct - Growth</t>
         </is>
       </c>
       <c r="C76" s="12" t="n">
-        <v>74.90000000000001</v>
+        <v>75.3</v>
       </c>
       <c r="D76" s="5" t="n">
-        <v>24.13</v>
+        <v>29.42</v>
       </c>
       <c r="E76" s="5" t="n">
-        <v>16.25</v>
+        <v>17.65</v>
       </c>
       <c r="F76" s="5" t="n">
-        <v>1.56</v>
-      </c>
-      <c r="G76" s="6" t="n">
-        <v>-34.67</v>
+        <v>1.59</v>
+      </c>
+      <c r="G76" s="5" t="n">
+        <v>-27.61</v>
       </c>
       <c r="H76" s="7" t="n">
-        <v>26.15</v>
+        <v>34.52</v>
       </c>
     </row>
     <row r="78">
@@ -7565,80 +7565,78 @@
       </c>
       <c r="B7" s="8" t="inlineStr">
         <is>
-          <t>Invesco India - Invesco Global Equity Income Fund of Fund - Direct Plan - Growth</t>
+          <t>DSP Global Innovation Overseas Equity Omni FoF - Direct - Growth</t>
         </is>
       </c>
       <c r="C7" s="28" t="n">
-        <v>74.90000000000001</v>
+        <v>75.3</v>
       </c>
       <c r="D7" s="11" t="n">
-        <v>19.24</v>
+        <v>19.44</v>
       </c>
       <c r="E7" s="11" t="n">
-        <v>24.13</v>
+        <v>29.42</v>
       </c>
       <c r="F7" s="11" t="n">
-        <v>16.25</v>
+        <v>17.65</v>
       </c>
       <c r="G7" s="11" t="n">
-        <v>14.6</v>
+        <v>8.470000000000001</v>
       </c>
       <c r="H7" s="11" t="n">
-        <v>20.69</v>
+        <v>25.04</v>
       </c>
       <c r="I7" s="11" t="n">
-        <v>20.18</v>
+        <v>25.32</v>
       </c>
       <c r="J7" s="11" t="n">
-        <v>13.1</v>
-      </c>
-      <c r="K7" s="11" t="n">
-        <v>12.32</v>
-      </c>
+        <v>27.42</v>
+      </c>
+      <c r="K7" s="13" t="n"/>
       <c r="L7" s="10" t="n">
-        <v>1.56</v>
+        <v>1.59</v>
       </c>
       <c r="M7" s="10" t="n">
-        <v>2.23</v>
+        <v>2.15</v>
       </c>
       <c r="N7" s="10" t="n">
-        <v>14.6</v>
+        <v>18.69</v>
       </c>
       <c r="O7" s="13" t="n">
-        <v>-34.67</v>
+        <v>-27.61</v>
       </c>
       <c r="P7" s="10" t="n">
-        <v>0.7</v>
+        <v>1.07</v>
       </c>
       <c r="Q7" s="10" t="n">
-        <v>-1.28</v>
+        <v>-1.67</v>
       </c>
       <c r="R7" s="17" t="n">
-        <v>43.5</v>
+        <v>31.5</v>
       </c>
       <c r="S7" s="17" t="n">
-        <v>48.6</v>
+        <v>19.6</v>
       </c>
       <c r="T7" s="11" t="n">
-        <v>26.15</v>
+        <v>34.52</v>
       </c>
       <c r="U7" s="18" t="n">
-        <v>0.431</v>
+        <v>0.226</v>
       </c>
       <c r="V7" s="18" t="n">
-        <v>0.155</v>
+        <v>0.026</v>
       </c>
       <c r="W7" s="11" t="n">
-        <v>1.3</v>
+        <v>1.21</v>
       </c>
       <c r="X7" s="17" t="n">
-        <v>81.8</v>
+        <v>95.8</v>
       </c>
       <c r="Y7" s="17" t="n">
-        <v>12.5</v>
+        <v>4.7</v>
       </c>
       <c r="Z7" s="8" t="n">
-        <v>41.4579</v>
+        <v>22.6584</v>
       </c>
     </row>
     <row r="8">
@@ -7647,78 +7645,80 @@
       </c>
       <c r="B8" s="19" t="inlineStr">
         <is>
-          <t>DSP Global Innovation Overseas Equity Omni FoF - Direct - Growth</t>
+          <t>Invesco India - Invesco Global Equity Income Fund of Fund - Direct Plan - Growth</t>
         </is>
       </c>
       <c r="C8" s="29" t="n">
-        <v>74.40000000000001</v>
+        <v>74.90000000000001</v>
       </c>
       <c r="D8" s="21" t="n">
-        <v>20.4</v>
+        <v>19.24</v>
       </c>
       <c r="E8" s="21" t="n">
-        <v>27.53</v>
+        <v>24.13</v>
       </c>
       <c r="F8" s="21" t="n">
-        <v>17.56</v>
+        <v>16.25</v>
       </c>
       <c r="G8" s="21" t="n">
-        <v>8.43</v>
+        <v>14.6</v>
       </c>
       <c r="H8" s="21" t="n">
-        <v>24.77</v>
+        <v>20.69</v>
       </c>
       <c r="I8" s="21" t="n">
-        <v>25.23</v>
+        <v>20.18</v>
       </c>
       <c r="J8" s="21" t="n">
-        <v>27.47</v>
-      </c>
-      <c r="K8" s="23" t="n"/>
+        <v>13.1</v>
+      </c>
+      <c r="K8" s="21" t="n">
+        <v>12.32</v>
+      </c>
       <c r="L8" s="22" t="n">
-        <v>1.46</v>
+        <v>1.56</v>
       </c>
       <c r="M8" s="22" t="n">
-        <v>1.98</v>
+        <v>2.23</v>
       </c>
       <c r="N8" s="22" t="n">
-        <v>18.73</v>
+        <v>14.6</v>
       </c>
       <c r="O8" s="23" t="n">
-        <v>-27.61</v>
+        <v>-34.67</v>
       </c>
       <c r="P8" s="22" t="n">
-        <v>1</v>
+        <v>0.7</v>
       </c>
       <c r="Q8" s="22" t="n">
-        <v>-1.69</v>
+        <v>-1.28</v>
       </c>
       <c r="R8" s="24" t="n">
-        <v>31.5</v>
+        <v>43.5</v>
       </c>
       <c r="S8" s="24" t="n">
-        <v>23.1</v>
+        <v>48.6</v>
       </c>
       <c r="T8" s="21" t="n">
-        <v>32.19</v>
+        <v>26.15</v>
       </c>
       <c r="U8" s="25" t="n">
-        <v>0.231</v>
+        <v>0.431</v>
       </c>
       <c r="V8" s="25" t="n">
-        <v>0.027</v>
+        <v>0.155</v>
       </c>
       <c r="W8" s="21" t="n">
-        <v>1.13</v>
+        <v>1.3</v>
       </c>
       <c r="X8" s="24" t="n">
-        <v>95.8</v>
+        <v>81.8</v>
       </c>
       <c r="Y8" s="24" t="n">
-        <v>4.7</v>
+        <v>12.5</v>
       </c>
       <c r="Z8" s="19" t="n">
-        <v>22.5706</v>
+        <v>41.4579</v>
       </c>
     </row>
     <row r="9">
@@ -8141,76 +8141,76 @@
         </is>
       </c>
       <c r="C14" s="20" t="n">
-        <v>67.90000000000001</v>
+        <v>68.8</v>
       </c>
       <c r="D14" s="21" t="n">
-        <v>22.52</v>
+        <v>21.54</v>
       </c>
       <c r="E14" s="21" t="n">
-        <v>23.9</v>
+        <v>25.75</v>
       </c>
       <c r="F14" s="21" t="n">
-        <v>8.67</v>
+        <v>8.74</v>
       </c>
       <c r="G14" s="21" t="n">
-        <v>4.29</v>
+        <v>4.34</v>
       </c>
       <c r="H14" s="21" t="n">
-        <v>21.38</v>
+        <v>21.71</v>
       </c>
       <c r="I14" s="21" t="n">
-        <v>18.89</v>
+        <v>19.03</v>
       </c>
       <c r="J14" s="21" t="n">
-        <v>15.5</v>
+        <v>15.52</v>
       </c>
       <c r="K14" s="21" t="n">
-        <v>16.5</v>
+        <v>16.58</v>
       </c>
       <c r="L14" s="22" t="n">
-        <v>1.18</v>
+        <v>1.3</v>
       </c>
       <c r="M14" s="22" t="n">
-        <v>1.67</v>
+        <v>1.83</v>
       </c>
       <c r="N14" s="22" t="n">
-        <v>18.52</v>
+        <v>18.48</v>
       </c>
       <c r="O14" s="23" t="n">
         <v>-39.98</v>
       </c>
       <c r="P14" s="22" t="n">
-        <v>0.6</v>
+        <v>0.64</v>
       </c>
       <c r="Q14" s="22" t="n">
-        <v>-1.81</v>
+        <v>-1.79</v>
       </c>
       <c r="R14" s="24" t="n">
         <v>26.4</v>
       </c>
       <c r="S14" s="24" t="n">
-        <v>22.5</v>
+        <v>19.1</v>
       </c>
       <c r="T14" s="21" t="n">
-        <v>27.51</v>
+        <v>29.66</v>
       </c>
       <c r="U14" s="25" t="n">
-        <v>0.189</v>
+        <v>0.183</v>
       </c>
       <c r="V14" s="25" t="n">
-        <v>0.019</v>
+        <v>0.018</v>
       </c>
       <c r="W14" s="21" t="n">
-        <v>0.99</v>
+        <v>1.07</v>
       </c>
       <c r="X14" s="24" t="n">
-        <v>82.59999999999999</v>
+        <v>82.7</v>
       </c>
       <c r="Y14" s="24" t="n">
         <v>5.2</v>
       </c>
       <c r="Z14" s="19" t="n">
-        <v>15.2617</v>
+        <v>15.3349</v>
       </c>
     </row>
     <row r="15">
@@ -8223,67 +8223,67 @@
         </is>
       </c>
       <c r="C15" s="16" t="n">
-        <v>67.40000000000001</v>
+        <v>68.40000000000001</v>
       </c>
       <c r="D15" s="11" t="n">
-        <v>15.56</v>
+        <v>13.8</v>
       </c>
       <c r="E15" s="11" t="n">
-        <v>19.3</v>
+        <v>20.45</v>
       </c>
       <c r="F15" s="11" t="n">
-        <v>12.08</v>
+        <v>12.06</v>
       </c>
       <c r="G15" s="11" t="n">
-        <v>12.77</v>
+        <v>12.7</v>
       </c>
       <c r="H15" s="11" t="n">
-        <v>17.82</v>
+        <v>17.83</v>
       </c>
       <c r="I15" s="11" t="n">
-        <v>17.09</v>
+        <v>17.06</v>
       </c>
       <c r="J15" s="11" t="n">
         <v>10.37</v>
       </c>
       <c r="K15" s="11" t="n">
-        <v>9.470000000000001</v>
+        <v>9.49</v>
       </c>
       <c r="L15" s="10" t="n">
-        <v>1.2</v>
+        <v>1.31</v>
       </c>
       <c r="M15" s="10" t="n">
-        <v>1.62</v>
+        <v>1.76</v>
       </c>
       <c r="N15" s="10" t="n">
-        <v>13.22</v>
+        <v>13.19</v>
       </c>
       <c r="O15" s="13" t="n">
         <v>-30.06</v>
       </c>
       <c r="P15" s="10" t="n">
-        <v>0.64</v>
+        <v>0.68</v>
       </c>
       <c r="Q15" s="10" t="n">
-        <v>-1.33</v>
+        <v>-1.32</v>
       </c>
       <c r="R15" s="17" t="n">
         <v>17.6</v>
       </c>
       <c r="S15" s="17" t="n">
-        <v>13.3</v>
+        <v>10.9</v>
       </c>
       <c r="T15" s="11" t="n">
-        <v>21.7</v>
+        <v>23.05</v>
       </c>
       <c r="U15" s="18" t="n">
-        <v>0.152</v>
+        <v>0.148</v>
       </c>
       <c r="V15" s="18" t="n">
-        <v>0.024</v>
+        <v>0.023</v>
       </c>
       <c r="W15" s="11" t="n">
-        <v>0.95</v>
+        <v>1</v>
       </c>
       <c r="X15" s="17" t="n">
         <v>73.3</v>
@@ -8292,12 +8292,12 @@
         <v>13.8</v>
       </c>
       <c r="Z15" s="8" t="n">
-        <v>47.864</v>
+        <v>47.885</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="19" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B16" s="19" t="inlineStr">
         <is>
@@ -8305,46 +8305,46 @@
         </is>
       </c>
       <c r="C16" s="20" t="n">
-        <v>67.40000000000001</v>
+        <v>67.8</v>
       </c>
       <c r="D16" s="21" t="n">
-        <v>14.1</v>
+        <v>12.22</v>
       </c>
       <c r="E16" s="21" t="n">
-        <v>20.42</v>
+        <v>21.38</v>
       </c>
       <c r="F16" s="21" t="n">
-        <v>9.869999999999999</v>
+        <v>9.640000000000001</v>
       </c>
       <c r="G16" s="21" t="n">
-        <v>8.59</v>
+        <v>8.539999999999999</v>
       </c>
       <c r="H16" s="21" t="n">
-        <v>19.24</v>
+        <v>18.87</v>
       </c>
       <c r="I16" s="21" t="n">
-        <v>16.25</v>
+        <v>16</v>
       </c>
       <c r="J16" s="21" t="n">
-        <v>13.04</v>
+        <v>13.03</v>
       </c>
       <c r="K16" s="21" t="n">
-        <v>9.029999999999999</v>
+        <v>9.09</v>
       </c>
       <c r="L16" s="22" t="n">
-        <v>1.26</v>
+        <v>1.34</v>
       </c>
       <c r="M16" s="22" t="n">
-        <v>1.64</v>
+        <v>1.74</v>
       </c>
       <c r="N16" s="22" t="n">
-        <v>14.31</v>
+        <v>14.29</v>
       </c>
       <c r="O16" s="23" t="n">
         <v>-27.06</v>
       </c>
       <c r="P16" s="22" t="n">
-        <v>0.75</v>
+        <v>0.79</v>
       </c>
       <c r="Q16" s="22" t="n">
         <v>-1.36</v>
@@ -8353,28 +8353,28 @@
         <v>31.2</v>
       </c>
       <c r="S16" s="24" t="n">
-        <v>38.1</v>
+        <v>36.6</v>
       </c>
       <c r="T16" s="21" t="n">
-        <v>21.95</v>
+        <v>23.09</v>
       </c>
       <c r="U16" s="25" t="n">
-        <v>0.353</v>
+        <v>0.351</v>
       </c>
       <c r="V16" s="25" t="n">
-        <v>0.108</v>
+        <v>0.107</v>
       </c>
       <c r="W16" s="21" t="n">
-        <v>1</v>
+        <v>1.06</v>
       </c>
       <c r="X16" s="24" t="n">
-        <v>79.90000000000001</v>
+        <v>80</v>
       </c>
       <c r="Y16" s="24" t="n">
         <v>7</v>
       </c>
       <c r="Z16" s="19" t="n">
-        <v>22.8269</v>
+        <v>22.7156</v>
       </c>
     </row>
     <row r="17">
@@ -8387,37 +8387,37 @@
         </is>
       </c>
       <c r="C17" s="16" t="n">
-        <v>67</v>
+        <v>67.09999999999999</v>
       </c>
       <c r="D17" s="11" t="n">
-        <v>25.68</v>
+        <v>25.26</v>
       </c>
       <c r="E17" s="11" t="n">
-        <v>24.58</v>
+        <v>25.51</v>
       </c>
       <c r="F17" s="11" t="n">
-        <v>10.33</v>
+        <v>9.92</v>
       </c>
       <c r="G17" s="11" t="n">
-        <v>11.19</v>
+        <v>11.1</v>
       </c>
       <c r="H17" s="11" t="n">
-        <v>26.43</v>
+        <v>25.91</v>
       </c>
       <c r="I17" s="11" t="n">
-        <v>19.74</v>
+        <v>19.42</v>
       </c>
       <c r="J17" s="11" t="n">
-        <v>10.5</v>
+        <v>10.52</v>
       </c>
       <c r="K17" s="11" t="n">
-        <v>7.31</v>
+        <v>7.35</v>
       </c>
       <c r="L17" s="10" t="n">
-        <v>1.19</v>
+        <v>1.25</v>
       </c>
       <c r="M17" s="10" t="n">
-        <v>1.46</v>
+        <v>1.53</v>
       </c>
       <c r="N17" s="10" t="n">
         <v>18.49</v>
@@ -8426,7 +8426,7 @@
         <v>-31.96</v>
       </c>
       <c r="P17" s="10" t="n">
-        <v>0.77</v>
+        <v>0.8</v>
       </c>
       <c r="Q17" s="10" t="n">
         <v>-1.81</v>
@@ -8435,28 +8435,28 @@
         <v>60.2</v>
       </c>
       <c r="S17" s="17" t="n">
-        <v>66.2</v>
+        <v>65.3</v>
       </c>
       <c r="T17" s="11" t="n">
-        <v>24.1</v>
+        <v>25.12</v>
       </c>
       <c r="U17" s="18" t="n">
-        <v>0.5570000000000001</v>
+        <v>0.556</v>
       </c>
       <c r="V17" s="18" t="n">
         <v>0.164</v>
       </c>
       <c r="W17" s="11" t="n">
-        <v>1.05</v>
+        <v>1.09</v>
       </c>
       <c r="X17" s="17" t="n">
-        <v>70.09999999999999</v>
+        <v>70.2</v>
       </c>
       <c r="Y17" s="17" t="n">
         <v>13.8</v>
       </c>
       <c r="Z17" s="8" t="n">
-        <v>40.62</v>
+        <v>40.368</v>
       </c>
     </row>
     <row r="18">
@@ -9613,38 +9613,38 @@
         </is>
       </c>
       <c r="C32" s="20" t="n">
-        <v>51</v>
+        <v>50.9</v>
       </c>
       <c r="D32" s="21" t="n">
-        <v>16.66</v>
+        <v>16.54</v>
       </c>
       <c r="E32" s="21" t="n">
-        <v>5.27</v>
+        <v>5.23</v>
       </c>
       <c r="F32" s="21" t="n">
-        <v>3.13</v>
+        <v>3.11</v>
       </c>
       <c r="G32" s="21" t="n">
-        <v>1.55</v>
+        <v>1.54</v>
       </c>
       <c r="H32" s="23" t="n"/>
       <c r="I32" s="23" t="n"/>
       <c r="J32" s="23" t="n"/>
       <c r="K32" s="23" t="n"/>
       <c r="L32" s="22" t="n">
-        <v>2.58</v>
+        <v>2.53</v>
       </c>
       <c r="M32" s="22" t="n">
-        <v>3.72</v>
+        <v>3.66</v>
       </c>
       <c r="N32" s="22" t="n">
-        <v>11.46</v>
+        <v>11.42</v>
       </c>
       <c r="O32" s="22" t="n">
         <v>-3.86</v>
       </c>
       <c r="P32" s="22" t="n">
-        <v>1.37</v>
+        <v>1.35</v>
       </c>
       <c r="Q32" s="22" t="n">
         <v>-0.88</v>
@@ -9653,26 +9653,26 @@
         <v>16.1</v>
       </c>
       <c r="S32" s="24" t="n">
-        <v>-15.4</v>
+        <v>-14.5</v>
       </c>
       <c r="T32" s="21" t="n">
-        <v>35.58</v>
+        <v>35.15</v>
       </c>
       <c r="U32" s="25" t="n">
-        <v>0.058</v>
+        <v>0.06</v>
       </c>
       <c r="V32" s="25" t="n">
         <v>0.005</v>
       </c>
       <c r="W32" s="21" t="n">
-        <v>1.5</v>
+        <v>1.61</v>
       </c>
       <c r="X32" s="24" t="n"/>
       <c r="Y32" s="24" t="n">
-        <v>0.5</v>
+        <v>0.6</v>
       </c>
       <c r="Z32" s="19" t="n">
-        <v>11.681</v>
+        <v>11.669</v>
       </c>
     </row>
     <row r="33">
@@ -32658,7 +32658,7 @@
         <v>6.93</v>
       </c>
       <c r="F76" s="21" t="n">
-        <v>4.51</v>
+        <v>4.52</v>
       </c>
       <c r="G76" s="21" t="n">
         <v>2.23</v>
@@ -32676,10 +32676,10 @@
         <v>7</v>
       </c>
       <c r="L76" s="22" t="n">
-        <v>-14.54</v>
+        <v>-14.55</v>
       </c>
       <c r="M76" s="22" t="n">
-        <v>-46.06</v>
+        <v>-46.08</v>
       </c>
       <c r="N76" s="22" t="n">
         <v>0.12</v>
@@ -32718,7 +32718,7 @@
         <v>3.3</v>
       </c>
       <c r="Z76" s="19" t="n">
-        <v>1247.2292</v>
+        <v>1247.4435</v>
       </c>
     </row>
     <row r="77">
@@ -33812,7 +33812,7 @@
         <v>6.05</v>
       </c>
       <c r="F91" s="11" t="n">
-        <v>3.98</v>
+        <v>3.99</v>
       </c>
       <c r="G91" s="11" t="n">
         <v>1.97</v>
@@ -33830,7 +33830,7 @@
         <v>6.14</v>
       </c>
       <c r="L91" s="10" t="n">
-        <v>-40.32</v>
+        <v>-40.34</v>
       </c>
       <c r="M91" s="10" t="n"/>
       <c r="N91" s="10" t="n">
@@ -33868,7 +33868,7 @@
         <v>3.3</v>
       </c>
       <c r="Z91" s="8" t="n">
-        <v>1215.907</v>
+        <v>1216.0946</v>
       </c>
     </row>
     <row r="92">
@@ -35732,44 +35732,44 @@
         </is>
       </c>
       <c r="C16" s="26" t="n">
-        <v>31.1</v>
+        <v>30.4</v>
       </c>
       <c r="D16" s="23" t="n">
-        <v>-5.04</v>
+        <v>-6.22</v>
       </c>
       <c r="E16" s="21" t="n">
-        <v>3.52</v>
+        <v>3.04</v>
       </c>
       <c r="F16" s="21" t="n">
-        <v>2.1</v>
+        <v>1.81</v>
       </c>
       <c r="G16" s="21" t="n">
-        <v>1.04</v>
-      </c>
-      <c r="H16" s="21" t="n">
-        <v>0.03</v>
-      </c>
-      <c r="I16" s="21" t="n">
-        <v>0.03</v>
+        <v>0.9</v>
+      </c>
+      <c r="H16" s="23" t="n">
+        <v>-1.01</v>
+      </c>
+      <c r="I16" s="23" t="n">
+        <v>-1.01</v>
       </c>
       <c r="J16" s="23" t="n">
-        <v>-3.43</v>
+        <v>-3.47</v>
       </c>
       <c r="K16" s="23" t="n"/>
       <c r="L16" s="22" t="n">
-        <v>-0.05</v>
+        <v>-0.08</v>
       </c>
       <c r="M16" s="22" t="n">
-        <v>-0.07000000000000001</v>
+        <v>-0.12</v>
       </c>
       <c r="N16" s="22" t="n">
-        <v>17.03</v>
+        <v>17.04</v>
       </c>
       <c r="O16" s="23" t="n">
         <v>-28.59</v>
       </c>
       <c r="P16" s="22" t="n">
-        <v>0.12</v>
+        <v>0.11</v>
       </c>
       <c r="Q16" s="22" t="n">
         <v>-1.66</v>
@@ -35778,28 +35778,28 @@
         <v>83.59999999999999</v>
       </c>
       <c r="S16" s="24" t="n">
-        <v>94</v>
+        <v>94.09999999999999</v>
       </c>
       <c r="T16" s="21" t="n">
-        <v>3.13</v>
+        <v>2.95</v>
       </c>
       <c r="U16" s="25" t="n">
-        <v>0.857</v>
+        <v>0.858</v>
       </c>
       <c r="V16" s="25" t="n">
-        <v>0.471</v>
+        <v>0.472</v>
       </c>
       <c r="W16" s="21" t="n">
-        <v>0.21</v>
+        <v>0.2</v>
       </c>
       <c r="X16" s="24" t="n">
-        <v>25</v>
+        <v>24.7</v>
       </c>
       <c r="Y16" s="24" t="n">
         <v>2.6</v>
       </c>
       <c r="Z16" s="19" t="n">
-        <v>11.114</v>
+        <v>10.96</v>
       </c>
     </row>
   </sheetData>
@@ -41996,46 +41996,46 @@
         </is>
       </c>
       <c r="C3" s="16" t="n">
-        <v>65.90000000000001</v>
+        <v>65.59999999999999</v>
       </c>
       <c r="D3" s="13" t="n">
-        <v>-1.81</v>
+        <v>-3.24</v>
       </c>
       <c r="E3" s="11" t="n">
-        <v>13.09</v>
+        <v>13.03</v>
       </c>
       <c r="F3" s="11" t="n">
         <v>12.01</v>
       </c>
       <c r="G3" s="11" t="n">
-        <v>15.11</v>
+        <v>15</v>
       </c>
       <c r="H3" s="11" t="n">
-        <v>6.59</v>
+        <v>5.95</v>
       </c>
       <c r="I3" s="11" t="n">
-        <v>12.09</v>
+        <v>11.69</v>
       </c>
       <c r="J3" s="11" t="n">
-        <v>17.84</v>
+        <v>17.8</v>
       </c>
       <c r="K3" s="11" t="n">
-        <v>17.22</v>
+        <v>17.21</v>
       </c>
       <c r="L3" s="10" t="n">
         <v>0.76</v>
       </c>
       <c r="M3" s="10" t="n">
-        <v>1.04</v>
+        <v>1.03</v>
       </c>
       <c r="N3" s="10" t="n">
-        <v>10.27</v>
+        <v>10.3</v>
       </c>
       <c r="O3" s="13" t="n">
         <v>-35.74</v>
       </c>
       <c r="P3" s="10" t="n">
-        <v>0.37</v>
+        <v>0.36</v>
       </c>
       <c r="Q3" s="10" t="n">
         <v>-1.09</v>
@@ -42044,10 +42044,10 @@
         <v>61.5</v>
       </c>
       <c r="S3" s="17" t="n">
-        <v>79.7</v>
+        <v>79.90000000000001</v>
       </c>
       <c r="T3" s="11" t="n">
-        <v>9.41</v>
+        <v>9.31</v>
       </c>
       <c r="U3" s="18" t="n">
         <v>0.699</v>
@@ -42056,16 +42056,16 @@
         <v>0.791</v>
       </c>
       <c r="W3" s="11" t="n">
-        <v>1.16</v>
+        <v>1.14</v>
       </c>
       <c r="X3" s="17" t="n">
-        <v>89.7</v>
+        <v>89.5</v>
       </c>
       <c r="Y3" s="17" t="n">
         <v>13.5</v>
       </c>
       <c r="Z3" s="8" t="n">
-        <v>240.6479</v>
+        <v>238.4188</v>
       </c>
     </row>
     <row r="4">
@@ -45131,80 +45131,80 @@
       </c>
       <c r="B8" s="19" t="inlineStr">
         <is>
-          <t>ICICI Prudential Dynamic Asset Allocation Active FOF - Direct Plan - Growth</t>
+          <t>Aditya Birla Sun Life Balanced Advantage Fund - Direct Plan - Growth Option</t>
         </is>
       </c>
       <c r="C8" s="20" t="n">
-        <v>59</v>
-      </c>
-      <c r="D8" s="23" t="n">
-        <v>-0.05</v>
+        <v>58.8</v>
+      </c>
+      <c r="D8" s="21" t="n">
+        <v>2.88</v>
       </c>
       <c r="E8" s="21" t="n">
-        <v>10.13</v>
+        <v>11.37</v>
       </c>
       <c r="F8" s="21" t="n">
-        <v>10.19</v>
+        <v>9.51</v>
       </c>
       <c r="G8" s="21" t="n">
-        <v>11.94</v>
+        <v>10.64</v>
       </c>
       <c r="H8" s="21" t="n">
-        <v>5.82</v>
+        <v>7.43</v>
       </c>
       <c r="I8" s="21" t="n">
-        <v>9.470000000000001</v>
+        <v>10.02</v>
       </c>
       <c r="J8" s="21" t="n">
-        <v>13.42</v>
+        <v>11.89</v>
       </c>
       <c r="K8" s="21" t="n">
-        <v>13.13</v>
+        <v>11.85</v>
       </c>
       <c r="L8" s="22" t="n">
-        <v>0.68</v>
+        <v>0.67</v>
       </c>
       <c r="M8" s="22" t="n">
-        <v>0.91</v>
+        <v>0.87</v>
       </c>
       <c r="N8" s="22" t="n">
-        <v>6.42</v>
+        <v>8.359999999999999</v>
       </c>
       <c r="O8" s="23" t="n">
-        <v>-26.35</v>
+        <v>-26.36</v>
       </c>
       <c r="P8" s="22" t="n">
-        <v>0.38</v>
+        <v>0.43</v>
       </c>
       <c r="Q8" s="22" t="n">
-        <v>-0.61</v>
+        <v>-0.78</v>
       </c>
       <c r="R8" s="24" t="n">
-        <v>30.6</v>
+        <v>43.3</v>
       </c>
       <c r="S8" s="24" t="n">
-        <v>56.4</v>
+        <v>69.90000000000001</v>
       </c>
       <c r="T8" s="21" t="n">
-        <v>7.7</v>
+        <v>7.55</v>
       </c>
       <c r="U8" s="25" t="n">
-        <v>0.429</v>
+        <v>0.589</v>
       </c>
       <c r="V8" s="25" t="n">
-        <v>0.764</v>
+        <v>0.894</v>
       </c>
       <c r="W8" s="21" t="n">
-        <v>0.44</v>
+        <v>0.71</v>
       </c>
       <c r="X8" s="24" t="n">
-        <v>95.90000000000001</v>
+        <v>94.09999999999999</v>
       </c>
       <c r="Y8" s="24" t="n">
-        <v>13.8</v>
+        <v>12</v>
       </c>
       <c r="Z8" s="19" t="n">
-        <v>136.1238</v>
+        <v>127.17</v>
       </c>
     </row>
     <row r="9">
@@ -45213,80 +45213,80 @@
       </c>
       <c r="B9" s="8" t="inlineStr">
         <is>
-          <t>Aditya Birla Sun Life Balanced Advantage Fund - Direct Plan - Growth Option</t>
+          <t>SBI Balanced Advantage Fund - Direct Plan - Growth</t>
         </is>
       </c>
       <c r="C9" s="16" t="n">
-        <v>58.8</v>
-      </c>
-      <c r="D9" s="11" t="n">
-        <v>2.88</v>
+        <v>58.5</v>
+      </c>
+      <c r="D9" s="13" t="n">
+        <v>-1.62</v>
       </c>
       <c r="E9" s="11" t="n">
-        <v>11.37</v>
+        <v>9.210000000000001</v>
       </c>
       <c r="F9" s="11" t="n">
-        <v>9.51</v>
+        <v>9.449999999999999</v>
       </c>
       <c r="G9" s="11" t="n">
-        <v>10.64</v>
+        <v>4.83</v>
       </c>
       <c r="H9" s="11" t="n">
-        <v>7.43</v>
+        <v>3.86</v>
       </c>
       <c r="I9" s="11" t="n">
-        <v>10.02</v>
+        <v>8.26</v>
       </c>
       <c r="J9" s="11" t="n">
-        <v>11.89</v>
+        <v>12.47</v>
       </c>
       <c r="K9" s="11" t="n">
-        <v>11.85</v>
+        <v>13.79</v>
       </c>
       <c r="L9" s="10" t="n">
-        <v>0.67</v>
+        <v>0.46</v>
       </c>
       <c r="M9" s="10" t="n">
-        <v>0.87</v>
+        <v>0.58</v>
       </c>
       <c r="N9" s="10" t="n">
-        <v>8.359999999999999</v>
-      </c>
-      <c r="O9" s="13" t="n">
-        <v>-26.36</v>
+        <v>6.88</v>
+      </c>
+      <c r="O9" s="10" t="n">
+        <v>-7.39</v>
       </c>
       <c r="P9" s="10" t="n">
-        <v>0.43</v>
+        <v>1.25</v>
       </c>
       <c r="Q9" s="10" t="n">
-        <v>-0.78</v>
+        <v>-0.72</v>
       </c>
       <c r="R9" s="17" t="n">
-        <v>43.3</v>
+        <v>31.7</v>
       </c>
       <c r="S9" s="17" t="n">
-        <v>69.90000000000001</v>
+        <v>60.5</v>
       </c>
       <c r="T9" s="11" t="n">
-        <v>7.55</v>
+        <v>6.15</v>
       </c>
       <c r="U9" s="18" t="n">
-        <v>0.589</v>
+        <v>0.471</v>
       </c>
       <c r="V9" s="18" t="n">
-        <v>0.894</v>
+        <v>0.835</v>
       </c>
       <c r="W9" s="11" t="n">
-        <v>0.71</v>
+        <v>0.29</v>
       </c>
       <c r="X9" s="17" t="n">
-        <v>94.09999999999999</v>
+        <v>98.09999999999999</v>
       </c>
       <c r="Y9" s="17" t="n">
-        <v>12</v>
+        <v>5.1</v>
       </c>
       <c r="Z9" s="8" t="n">
-        <v>127.17</v>
+        <v>16.1116</v>
       </c>
     </row>
     <row r="10">
@@ -45295,80 +45295,80 @@
       </c>
       <c r="B10" s="19" t="inlineStr">
         <is>
-          <t>SBI Balanced Advantage Fund - Direct Plan - Growth</t>
+          <t>ICICI Prudential Dynamic Asset Allocation Active FOF - Direct Plan - Growth</t>
         </is>
       </c>
       <c r="C10" s="20" t="n">
-        <v>58.5</v>
+        <v>58.4</v>
       </c>
       <c r="D10" s="23" t="n">
-        <v>-1.62</v>
+        <v>-1.04</v>
       </c>
       <c r="E10" s="21" t="n">
-        <v>9.210000000000001</v>
+        <v>9.93</v>
       </c>
       <c r="F10" s="21" t="n">
-        <v>9.449999999999999</v>
+        <v>10.11</v>
       </c>
       <c r="G10" s="21" t="n">
-        <v>4.83</v>
+        <v>11.85</v>
       </c>
       <c r="H10" s="21" t="n">
-        <v>3.86</v>
+        <v>5.28</v>
       </c>
       <c r="I10" s="21" t="n">
-        <v>8.26</v>
+        <v>9.130000000000001</v>
       </c>
       <c r="J10" s="21" t="n">
-        <v>12.47</v>
+        <v>13.39</v>
       </c>
       <c r="K10" s="21" t="n">
-        <v>13.79</v>
+        <v>13.12</v>
       </c>
       <c r="L10" s="22" t="n">
-        <v>0.46</v>
+        <v>0.65</v>
       </c>
       <c r="M10" s="22" t="n">
-        <v>0.58</v>
+        <v>0.87</v>
       </c>
       <c r="N10" s="22" t="n">
-        <v>6.88</v>
-      </c>
-      <c r="O10" s="22" t="n">
-        <v>-7.39</v>
+        <v>6.45</v>
+      </c>
+      <c r="O10" s="23" t="n">
+        <v>-26.35</v>
       </c>
       <c r="P10" s="22" t="n">
-        <v>1.25</v>
+        <v>0.38</v>
       </c>
       <c r="Q10" s="22" t="n">
-        <v>-0.72</v>
+        <v>-0.63</v>
       </c>
       <c r="R10" s="24" t="n">
-        <v>31.7</v>
+        <v>30.6</v>
       </c>
       <c r="S10" s="24" t="n">
-        <v>60.5</v>
+        <v>56.8</v>
       </c>
       <c r="T10" s="21" t="n">
-        <v>6.15</v>
+        <v>7.48</v>
       </c>
       <c r="U10" s="25" t="n">
-        <v>0.471</v>
+        <v>0.43</v>
       </c>
       <c r="V10" s="25" t="n">
-        <v>0.835</v>
+        <v>0.764</v>
       </c>
       <c r="W10" s="21" t="n">
-        <v>0.29</v>
+        <v>0.41</v>
       </c>
       <c r="X10" s="24" t="n">
-        <v>98.09999999999999</v>
+        <v>95.8</v>
       </c>
       <c r="Y10" s="24" t="n">
-        <v>5.1</v>
+        <v>13.8</v>
       </c>
       <c r="Z10" s="19" t="n">
-        <v>16.1116</v>
+        <v>135.0766</v>
       </c>
     </row>
     <row r="11">
@@ -51409,7 +51409,7 @@
         <v>-13.29</v>
       </c>
       <c r="M3" s="10" t="n">
-        <v>-29.39</v>
+        <v>-29.4</v>
       </c>
       <c r="N3" s="10" t="n">
         <v>0.13</v>
@@ -51448,7 +51448,7 @@
         <v>9.9</v>
       </c>
       <c r="Z3" s="8" t="n">
-        <v>3694.4529</v>
+        <v>3695.0902</v>
       </c>
     </row>
     <row r="4">
@@ -51571,7 +51571,7 @@
         <v>-13.94</v>
       </c>
       <c r="M5" s="10" t="n">
-        <v>-30.3</v>
+        <v>-30.31</v>
       </c>
       <c r="N5" s="10" t="n">
         <v>0.12</v>
@@ -51610,7 +51610,7 @@
         <v>13.8</v>
       </c>
       <c r="Z5" s="8" t="n">
-        <v>4509.9927</v>
+        <v>4510.7724</v>
       </c>
     </row>
     <row r="6">
@@ -51632,7 +51632,7 @@
         <v>6.89</v>
       </c>
       <c r="F6" s="21" t="n">
-        <v>6.37</v>
+        <v>6.38</v>
       </c>
       <c r="G6" s="21" t="n">
         <v>6.05</v>
@@ -51653,7 +51653,7 @@
         <v>-13.05</v>
       </c>
       <c r="M6" s="22" t="n">
-        <v>-29.91</v>
+        <v>-29.92</v>
       </c>
       <c r="N6" s="22" t="n">
         <v>0.13</v>
@@ -51692,7 +51692,7 @@
         <v>13.8</v>
       </c>
       <c r="Z6" s="19" t="n">
-        <v>5610.0543</v>
+        <v>5611.0048</v>
       </c>
     </row>
     <row r="7">
@@ -51701,7 +51701,7 @@
       </c>
       <c r="B7" s="8" t="inlineStr">
         <is>
-          <t>Kotak Liquid Fund - Direct Plan - Growth</t>
+          <t>LIC MF Liquid Fund-Direct Plan-Growth</t>
         </is>
       </c>
       <c r="C7" s="16" t="n">
@@ -51711,16 +51711,16 @@
         <v>6.47</v>
       </c>
       <c r="E7" s="11" t="n">
-        <v>6.91</v>
+        <v>6.9</v>
       </c>
       <c r="F7" s="11" t="n">
-        <v>6.39</v>
+        <v>6.38</v>
       </c>
       <c r="G7" s="11" t="n">
-        <v>6.07</v>
+        <v>6.12</v>
       </c>
       <c r="H7" s="11" t="n">
-        <v>6.69</v>
+        <v>6.67</v>
       </c>
       <c r="I7" s="11" t="n">
         <v>6.73</v>
@@ -51729,34 +51729,32 @@
         <v>55.31</v>
       </c>
       <c r="K7" s="11" t="n">
-        <v>8.59</v>
+        <v>8.640000000000001</v>
       </c>
       <c r="L7" s="10" t="n">
-        <v>-9.48</v>
-      </c>
-      <c r="M7" s="10" t="n">
-        <v>-23.16</v>
-      </c>
+        <v>-13.68</v>
+      </c>
+      <c r="M7" s="10" t="n"/>
       <c r="N7" s="10" t="n">
-        <v>0.16</v>
+        <v>0.13</v>
       </c>
       <c r="O7" s="10" t="n">
-        <v>-0.26</v>
+        <v>-0.16</v>
       </c>
       <c r="P7" s="10" t="n">
-        <v>26.58</v>
+        <v>43.12</v>
       </c>
       <c r="Q7" s="10" t="n">
         <v>0.01</v>
       </c>
       <c r="R7" s="17" t="n">
-        <v>1.4</v>
+        <v>1.3</v>
       </c>
       <c r="S7" s="17" t="n">
         <v>-6</v>
       </c>
       <c r="T7" s="11" t="n">
-        <v>4.83</v>
+        <v>4.79</v>
       </c>
       <c r="U7" s="18" t="n">
         <v>0.001</v>
@@ -51774,7 +51772,7 @@
         <v>13.8</v>
       </c>
       <c r="Z7" s="8" t="n">
-        <v>5772.3608</v>
+        <v>5187.2526</v>
       </c>
     </row>
     <row r="8">
@@ -51783,156 +51781,158 @@
       </c>
       <c r="B8" s="19" t="inlineStr">
         <is>
-          <t>LIC MF Liquid Fund-Direct Plan-Growth</t>
+          <t>ING Liquid Fund - Super Institutional Plan - Direct Plan - Growth Option</t>
         </is>
       </c>
       <c r="C8" s="20" t="n">
         <v>50.1</v>
       </c>
       <c r="D8" s="21" t="n">
-        <v>6.47</v>
+        <v>9.31</v>
       </c>
       <c r="E8" s="21" t="n">
-        <v>6.9</v>
+        <v>5.38</v>
       </c>
       <c r="F8" s="21" t="n">
-        <v>6.38</v>
+        <v>3.19</v>
       </c>
       <c r="G8" s="21" t="n">
-        <v>6.12</v>
+        <v>1.58</v>
       </c>
       <c r="H8" s="21" t="n">
-        <v>6.67</v>
+        <v>9.300000000000001</v>
       </c>
       <c r="I8" s="21" t="n">
-        <v>6.73</v>
+        <v>9.300000000000001</v>
       </c>
       <c r="J8" s="21" t="n">
-        <v>55.31</v>
-      </c>
-      <c r="K8" s="21" t="n">
-        <v>8.640000000000001</v>
-      </c>
+        <v>9.52</v>
+      </c>
+      <c r="K8" s="23" t="n"/>
       <c r="L8" s="22" t="n">
-        <v>-13.67</v>
+        <v>3.16</v>
       </c>
       <c r="M8" s="22" t="n"/>
       <c r="N8" s="22" t="n">
-        <v>0.13</v>
+        <v>0.35</v>
       </c>
       <c r="O8" s="22" t="n">
-        <v>-0.16</v>
+        <v>-0.34</v>
       </c>
       <c r="P8" s="22" t="n">
-        <v>43.12</v>
+        <v>15.82</v>
       </c>
       <c r="Q8" s="22" t="n">
-        <v>0.01</v>
+        <v>0.02</v>
       </c>
       <c r="R8" s="24" t="n">
-        <v>1.3</v>
+        <v>1.2</v>
       </c>
       <c r="S8" s="24" t="n">
-        <v>-6</v>
+        <v>-7</v>
       </c>
       <c r="T8" s="21" t="n">
-        <v>4.79</v>
+        <v>6.3</v>
       </c>
       <c r="U8" s="25" t="n">
-        <v>0.001</v>
+        <v>0.003</v>
       </c>
       <c r="V8" s="25" t="n">
-        <v>0.005</v>
+        <v>0.015</v>
       </c>
       <c r="W8" s="23" t="n">
-        <v>-0.18</v>
+        <v>-0.82</v>
       </c>
       <c r="X8" s="24" t="n">
         <v>100</v>
       </c>
       <c r="Y8" s="24" t="n">
-        <v>13.8</v>
+        <v>1.8</v>
       </c>
       <c r="Z8" s="19" t="n">
-        <v>5186.3587</v>
+        <v>20.009</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="8" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="B9" s="8" t="inlineStr">
         <is>
-          <t>ING Liquid Fund - Super Institutional Plan - Direct Plan - Growth Option</t>
+          <t>Kotak Liquid Fund - Direct Plan - Growth</t>
         </is>
       </c>
       <c r="C9" s="16" t="n">
-        <v>50.1</v>
+        <v>50</v>
       </c>
       <c r="D9" s="11" t="n">
-        <v>9.31</v>
+        <v>6.47</v>
       </c>
       <c r="E9" s="11" t="n">
-        <v>5.38</v>
+        <v>6.9</v>
       </c>
       <c r="F9" s="11" t="n">
-        <v>3.19</v>
+        <v>6.39</v>
       </c>
       <c r="G9" s="11" t="n">
-        <v>1.58</v>
+        <v>6.07</v>
       </c>
       <c r="H9" s="11" t="n">
-        <v>9.300000000000001</v>
+        <v>6.69</v>
       </c>
       <c r="I9" s="11" t="n">
-        <v>9.300000000000001</v>
+        <v>6.73</v>
       </c>
       <c r="J9" s="11" t="n">
-        <v>9.52</v>
-      </c>
-      <c r="K9" s="13" t="n"/>
+        <v>55.31</v>
+      </c>
+      <c r="K9" s="11" t="n">
+        <v>8.59</v>
+      </c>
       <c r="L9" s="10" t="n">
-        <v>3.16</v>
-      </c>
-      <c r="M9" s="10" t="n"/>
+        <v>-9.529999999999999</v>
+      </c>
+      <c r="M9" s="10" t="n">
+        <v>-23.24</v>
+      </c>
       <c r="N9" s="10" t="n">
-        <v>0.35</v>
+        <v>0.16</v>
       </c>
       <c r="O9" s="10" t="n">
-        <v>-0.34</v>
+        <v>-0.26</v>
       </c>
       <c r="P9" s="10" t="n">
-        <v>15.82</v>
+        <v>26.54</v>
       </c>
       <c r="Q9" s="10" t="n">
-        <v>0.02</v>
+        <v>0.01</v>
       </c>
       <c r="R9" s="17" t="n">
-        <v>1.2</v>
+        <v>1.4</v>
       </c>
       <c r="S9" s="17" t="n">
-        <v>-7</v>
+        <v>-6</v>
       </c>
       <c r="T9" s="11" t="n">
-        <v>6.3</v>
+        <v>4.83</v>
       </c>
       <c r="U9" s="18" t="n">
-        <v>0.003</v>
+        <v>0.001</v>
       </c>
       <c r="V9" s="18" t="n">
-        <v>0.015</v>
+        <v>0.005</v>
       </c>
       <c r="W9" s="13" t="n">
-        <v>-0.82</v>
+        <v>-0.18</v>
       </c>
       <c r="X9" s="17" t="n">
         <v>100</v>
       </c>
       <c r="Y9" s="17" t="n">
-        <v>1.8</v>
+        <v>13.8</v>
       </c>
       <c r="Z9" s="8" t="n">
-        <v>20.009</v>
+        <v>5773.3782</v>
       </c>
     </row>
     <row r="10">
@@ -52408,7 +52408,7 @@
         <v>13.8</v>
       </c>
       <c r="Z15" s="8" t="n">
-        <v>461.741</v>
+        <v>461.8237</v>
       </c>
     </row>
     <row r="16">
@@ -52424,7 +52424,7 @@
         <v>46.5</v>
       </c>
       <c r="D16" s="21" t="n">
-        <v>6.56</v>
+        <v>6.57</v>
       </c>
       <c r="E16" s="21" t="n">
         <v>6.97</v>
@@ -52488,7 +52488,7 @@
         <v>13.8</v>
       </c>
       <c r="Z16" s="19" t="n">
-        <v>3179.971</v>
+        <v>3180.5188</v>
       </c>
     </row>
     <row r="17">
@@ -52595,7 +52595,7 @@
         <v>6.42</v>
       </c>
       <c r="G18" s="21" t="n">
-        <v>6.17</v>
+        <v>6.16</v>
       </c>
       <c r="H18" s="21" t="n">
         <v>6.75</v>
@@ -52650,7 +52650,7 @@
         <v>13.8</v>
       </c>
       <c r="Z18" s="19" t="n">
-        <v>4296.8361</v>
+        <v>4297.5732</v>
       </c>
     </row>
     <row r="19">
@@ -52672,7 +52672,7 @@
         <v>6.95</v>
       </c>
       <c r="F19" s="11" t="n">
-        <v>6.42</v>
+        <v>6.43</v>
       </c>
       <c r="G19" s="11" t="n">
         <v>6.15</v>
@@ -52693,7 +52693,7 @@
         <v>-13.24</v>
       </c>
       <c r="M19" s="10" t="n">
-        <v>-30.36</v>
+        <v>-30.37</v>
       </c>
       <c r="N19" s="10" t="n">
         <v>0.13</v>
@@ -52732,7 +52732,7 @@
         <v>13.8</v>
       </c>
       <c r="Z19" s="8" t="n">
-        <v>6996.7255</v>
+        <v>6997.9382</v>
       </c>
     </row>
     <row r="20">
@@ -52757,7 +52757,7 @@
         <v>6.31</v>
       </c>
       <c r="G20" s="21" t="n">
-        <v>6.04</v>
+        <v>6.03</v>
       </c>
       <c r="H20" s="21" t="n">
         <v>6.72</v>
@@ -52814,7 +52814,7 @@
         <v>13.8</v>
       </c>
       <c r="Z20" s="19" t="n">
-        <v>2770.2658</v>
+        <v>2770.7308</v>
       </c>
     </row>
     <row r="21">
@@ -52919,7 +52919,7 @@
         <v>6.41</v>
       </c>
       <c r="G22" s="21" t="n">
-        <v>6.11</v>
+        <v>6.1</v>
       </c>
       <c r="H22" s="21" t="n">
         <v>6.69</v>
@@ -52974,7 +52974,7 @@
         <v>13.8</v>
       </c>
       <c r="Z22" s="19" t="n">
-        <v>2846.689</v>
+        <v>2847.1848</v>
       </c>
     </row>
     <row r="23">
@@ -53017,7 +53017,7 @@
         <v>-13.7</v>
       </c>
       <c r="M23" s="10" t="n">
-        <v>-38.33</v>
+        <v>-38.34</v>
       </c>
       <c r="N23" s="10" t="n">
         <v>0.13</v>
@@ -53056,7 +53056,7 @@
         <v>13.8</v>
       </c>
       <c r="Z23" s="8" t="n">
-        <v>422.7574</v>
+        <v>422.8296</v>
       </c>
     </row>
     <row r="24">
@@ -53220,7 +53220,7 @@
         <v>13.8</v>
       </c>
       <c r="Z25" s="8" t="n">
-        <v>3016.113</v>
+        <v>3016.6418</v>
       </c>
     </row>
     <row r="26">
@@ -53263,7 +53263,7 @@
         <v>-13.89</v>
       </c>
       <c r="M26" s="22" t="n">
-        <v>-25.51</v>
+        <v>-25.52</v>
       </c>
       <c r="N26" s="22" t="n">
         <v>0.12</v>
@@ -53302,7 +53302,7 @@
         <v>13.8</v>
       </c>
       <c r="Z26" s="19" t="n">
-        <v>3424.1806</v>
+        <v>3424.7787</v>
       </c>
     </row>
     <row r="27">
@@ -53324,7 +53324,7 @@
         <v>6.87</v>
       </c>
       <c r="F27" s="11" t="n">
-        <v>6.36</v>
+        <v>6.37</v>
       </c>
       <c r="G27" s="11" t="n">
         <v>6.06</v>
@@ -53345,7 +53345,7 @@
         <v>-13.93</v>
       </c>
       <c r="M27" s="10" t="n">
-        <v>-37.73</v>
+        <v>-37.74</v>
       </c>
       <c r="N27" s="10" t="n">
         <v>0.13</v>
@@ -53384,7 +53384,7 @@
         <v>13.8</v>
       </c>
       <c r="Z27" s="8" t="n">
-        <v>4466.1092</v>
+        <v>4466.8604</v>
       </c>
     </row>
     <row r="28">
@@ -53427,7 +53427,7 @@
         <v>-13.83</v>
       </c>
       <c r="M28" s="22" t="n">
-        <v>-43.83</v>
+        <v>-43.84</v>
       </c>
       <c r="N28" s="22" t="n">
         <v>0.13</v>
@@ -53466,7 +53466,7 @@
         <v>13.8</v>
       </c>
       <c r="Z28" s="19" t="n">
-        <v>3449.6928</v>
+        <v>3450.2919</v>
       </c>
     </row>
     <row r="29">
@@ -53485,13 +53485,13 @@
         <v>6.39</v>
       </c>
       <c r="E29" s="11" t="n">
-        <v>6.83</v>
+        <v>6.82</v>
       </c>
       <c r="F29" s="11" t="n">
         <v>6.35</v>
       </c>
       <c r="G29" s="11" t="n">
-        <v>6.08</v>
+        <v>6.07</v>
       </c>
       <c r="H29" s="11" t="n">
         <v>6.6</v>
@@ -53506,7 +53506,7 @@
         <v>6.52</v>
       </c>
       <c r="L29" s="10" t="n">
-        <v>-7.93</v>
+        <v>-7.98</v>
       </c>
       <c r="M29" s="10" t="n"/>
       <c r="N29" s="10" t="n">
@@ -53516,7 +53516,7 @@
         <v>-0.18</v>
       </c>
       <c r="P29" s="10" t="n">
-        <v>37.94</v>
+        <v>37.89</v>
       </c>
       <c r="Q29" s="10" t="n">
         <v>0.01</v>
@@ -53546,7 +53546,7 @@
         <v>13.8</v>
       </c>
       <c r="Z29" s="8" t="n">
-        <v>77.9366</v>
+        <v>77.95010000000001</v>
       </c>
     </row>
     <row r="30">
@@ -53568,7 +53568,7 @@
         <v>6.93</v>
       </c>
       <c r="F30" s="21" t="n">
-        <v>6.42</v>
+        <v>6.43</v>
       </c>
       <c r="G30" s="21" t="n">
         <v>5.73</v>
@@ -53626,7 +53626,7 @@
         <v>13.8</v>
       </c>
       <c r="Z30" s="19" t="n">
-        <v>2756.0574</v>
+        <v>2756.537</v>
       </c>
     </row>
     <row r="31">
@@ -53746,7 +53746,7 @@
         <v>5.96</v>
       </c>
       <c r="L32" s="22" t="n">
-        <v>-13.09</v>
+        <v>-13.1</v>
       </c>
       <c r="M32" s="22" t="n"/>
       <c r="N32" s="22" t="n">
@@ -53786,7 +53786,7 @@
         <v>10.6</v>
       </c>
       <c r="Z32" s="19" t="n">
-        <v>372.881</v>
+        <v>372.9442</v>
       </c>
     </row>
     <row r="33">
@@ -53805,13 +53805,13 @@
         <v>6.26</v>
       </c>
       <c r="E33" s="11" t="n">
-        <v>6.72</v>
+        <v>6.71</v>
       </c>
       <c r="F33" s="11" t="n">
         <v>6.22</v>
       </c>
       <c r="G33" s="11" t="n">
-        <v>5.73</v>
+        <v>5.72</v>
       </c>
       <c r="H33" s="11" t="n">
         <v>6.48</v>
@@ -53826,10 +53826,10 @@
         <v>5.9</v>
       </c>
       <c r="L33" s="10" t="n">
-        <v>-5.09</v>
+        <v>-5.13</v>
       </c>
       <c r="M33" s="10" t="n">
-        <v>-10.92</v>
+        <v>-10.99</v>
       </c>
       <c r="N33" s="10" t="n">
         <v>0.18</v>
@@ -53838,7 +53838,7 @@
         <v>-0.04</v>
       </c>
       <c r="P33" s="10" t="n">
-        <v>168</v>
+        <v>167.75</v>
       </c>
       <c r="Q33" s="10" t="n">
         <v>0.01</v>
@@ -53868,7 +53868,7 @@
         <v>12.9</v>
       </c>
       <c r="Z33" s="8" t="n">
-        <v>2186.0469</v>
+        <v>2186.4001</v>
       </c>
     </row>
     <row r="34">
@@ -53911,7 +53911,7 @@
         <v>-12.77</v>
       </c>
       <c r="M34" s="22" t="n">
-        <v>-28.36</v>
+        <v>-28.37</v>
       </c>
       <c r="N34" s="22" t="n">
         <v>0.13</v>
@@ -53950,7 +53950,7 @@
         <v>4.8</v>
       </c>
       <c r="Z34" s="19" t="n">
-        <v>2526.4207</v>
+        <v>2526.8618</v>
       </c>
     </row>
     <row r="35">
@@ -54049,7 +54049,7 @@
         <v>6.43</v>
       </c>
       <c r="E36" s="21" t="n">
-        <v>6.86</v>
+        <v>6.85</v>
       </c>
       <c r="F36" s="21" t="n">
         <v>6.36</v>
@@ -54070,7 +54070,7 @@
         <v>6.66</v>
       </c>
       <c r="L36" s="22" t="n">
-        <v>-11.83</v>
+        <v>-11.9</v>
       </c>
       <c r="M36" s="22" t="n"/>
       <c r="N36" s="22" t="n">
@@ -54080,7 +54080,7 @@
         <v>-0.01</v>
       </c>
       <c r="P36" s="22" t="n">
-        <v>686</v>
+        <v>685</v>
       </c>
       <c r="Q36" s="22" t="n">
         <v>0.01</v>
@@ -54110,7 +54110,7 @@
         <v>5.5</v>
       </c>
       <c r="Z36" s="19" t="n">
-        <v>1382.8894</v>
+        <v>1383.1224</v>
       </c>
     </row>
     <row r="37">
@@ -54535,7 +54535,7 @@
         <v>6.06</v>
       </c>
       <c r="E42" s="21" t="n">
-        <v>6.72</v>
+        <v>6.71</v>
       </c>
       <c r="F42" s="21" t="n">
         <v>6.31</v>
@@ -54556,7 +54556,7 @@
         <v>6.83</v>
       </c>
       <c r="L42" s="22" t="n">
-        <v>-5.6</v>
+        <v>-5.64</v>
       </c>
       <c r="M42" s="22" t="n"/>
       <c r="N42" s="22" t="n">
@@ -54596,7 +54596,7 @@
         <v>13.8</v>
       </c>
       <c r="Z42" s="19" t="n">
-        <v>45.728</v>
+        <v>45.7353</v>
       </c>
     </row>
     <row r="43">
@@ -54940,10 +54940,10 @@
         <v>40.9</v>
       </c>
       <c r="D47" s="11" t="n">
-        <v>6.55</v>
+        <v>6.56</v>
       </c>
       <c r="E47" s="11" t="n">
-        <v>2.69</v>
+        <v>2.7</v>
       </c>
       <c r="F47" s="11" t="n">
         <v>1.61</v>
@@ -54962,7 +54962,7 @@
       </c>
       <c r="K47" s="13" t="n"/>
       <c r="L47" s="10" t="n">
-        <v>-12.85</v>
+        <v>-12.87</v>
       </c>
       <c r="M47" s="10" t="n">
         <v>-32.82</v>
@@ -54974,7 +54974,7 @@
         <v>-0.01</v>
       </c>
       <c r="P47" s="10" t="n">
-        <v>269</v>
+        <v>270</v>
       </c>
       <c r="Q47" s="10" t="n">
         <v>0.01</v>
@@ -55004,7 +55004,7 @@
         <v>1.3</v>
       </c>
       <c r="Z47" s="8" t="n">
-        <v>1083.816</v>
+        <v>1084.0031</v>
       </c>
     </row>
     <row r="48">
@@ -55023,10 +55023,10 @@
         <v>6.32</v>
       </c>
       <c r="E48" s="21" t="n">
-        <v>4.02</v>
+        <v>4.03</v>
       </c>
       <c r="F48" s="21" t="n">
-        <v>2.39</v>
+        <v>2.4</v>
       </c>
       <c r="G48" s="21" t="n">
         <v>1.19</v>
@@ -55042,7 +55042,7 @@
       </c>
       <c r="K48" s="23" t="n"/>
       <c r="L48" s="22" t="n">
-        <v>-15.48</v>
+        <v>-15.49</v>
       </c>
       <c r="M48" s="22" t="n">
         <v>-34.32</v>
@@ -55054,7 +55054,7 @@
         <v>-0.01</v>
       </c>
       <c r="P48" s="22" t="n">
-        <v>402</v>
+        <v>403</v>
       </c>
       <c r="Q48" s="22" t="n">
         <v>0.01</v>
@@ -55084,7 +55084,7 @@
         <v>1.9</v>
       </c>
       <c r="Z48" s="19" t="n">
-        <v>1127.8941</v>
+        <v>1128.0858</v>
       </c>
     </row>
     <row r="49">
@@ -55335,19 +55335,19 @@
         <v>5.75</v>
       </c>
       <c r="E52" s="21" t="n">
-        <v>6.37</v>
+        <v>6.36</v>
       </c>
       <c r="F52" s="23" t="n">
         <v>-57.76</v>
       </c>
       <c r="G52" s="23" t="n">
-        <v>-33.18</v>
+        <v>-33.19</v>
       </c>
       <c r="H52" s="21" t="n">
         <v>6.09</v>
       </c>
       <c r="I52" s="23" t="n">
-        <v>-5.32</v>
+        <v>-5.31</v>
       </c>
       <c r="J52" s="21" t="n">
         <v>839.35</v>
@@ -55356,7 +55356,7 @@
         <v>46.64</v>
       </c>
       <c r="L52" s="22" t="n">
-        <v>-11.17</v>
+        <v>-11.23</v>
       </c>
       <c r="M52" s="22" t="n"/>
       <c r="N52" s="22" t="n">
@@ -55396,7 +55396,7 @@
         <v>13.8</v>
       </c>
       <c r="Z52" s="19" t="n">
-        <v>30.7944</v>
+        <v>30.7992</v>
       </c>
     </row>
     <row r="53">
@@ -55651,10 +55651,10 @@
         <v>6.54</v>
       </c>
       <c r="E56" s="21" t="n">
-        <v>2.15</v>
+        <v>2.16</v>
       </c>
       <c r="F56" s="21" t="n">
-        <v>1.28</v>
+        <v>1.29</v>
       </c>
       <c r="G56" s="21" t="n">
         <v>0.64</v>
@@ -55668,7 +55668,7 @@
       <c r="J56" s="23" t="n"/>
       <c r="K56" s="23" t="n"/>
       <c r="L56" s="22" t="n">
-        <v>-13.27</v>
+        <v>-13.29</v>
       </c>
       <c r="M56" s="22" t="n"/>
       <c r="N56" s="22" t="n">
@@ -55678,7 +55678,7 @@
         <v>-0.01</v>
       </c>
       <c r="P56" s="22" t="n">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="Q56" s="22" t="n">
         <v>0.01</v>
@@ -55706,7 +55706,7 @@
         <v>1</v>
       </c>
       <c r="Z56" s="19" t="n">
-        <v>1067.0307</v>
+        <v>1067.2101</v>
       </c>
     </row>
     <row r="57">
@@ -55722,7 +55722,7 @@
         <v>33.9</v>
       </c>
       <c r="D57" s="11" t="n">
-        <v>5.82</v>
+        <v>5.81</v>
       </c>
       <c r="E57" s="11" t="n">
         <v>2.61</v>
@@ -55731,7 +55731,7 @@
         <v>1.56</v>
       </c>
       <c r="G57" s="11" t="n">
-        <v>0.77</v>
+        <v>0.78</v>
       </c>
       <c r="H57" s="11" t="n">
         <v>5.77</v>
@@ -55744,7 +55744,7 @@
       </c>
       <c r="K57" s="13" t="n"/>
       <c r="L57" s="10" t="n">
-        <v>-16.53</v>
+        <v>-16.55</v>
       </c>
       <c r="M57" s="10" t="n"/>
       <c r="N57" s="10" t="n">
@@ -55782,7 +55782,7 @@
         <v>1.4</v>
       </c>
       <c r="Z57" s="8" t="n">
-        <v>1081.0121</v>
+        <v>1081.1622</v>
       </c>
     </row>
     <row r="58">
@@ -56555,7 +56555,7 @@
         <v>-13.7</v>
       </c>
       <c r="T3" s="11" t="n">
-        <v>8427847910015000</v>
+        <v>8427847910015416</v>
       </c>
       <c r="U3" s="18" t="n">
         <v>11.604</v>

</xml_diff>